<commit_message>
Manning plan: Fabiano bid (GW $30,500 + demo $7,400), GW at $25K target, Prime Seal roofing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY6xq9eh2BK6Au4SE2w7Bc
</commit_message>
<xml_diff>
--- a/Manning_Construction_Plan.xlsx
+++ b/Manning_Construction_Plan.xlsx
@@ -122,7 +122,19 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Renomar's approved bid covers General Works + Demo combined.</t>
+          <t xml:space="preserve">Renomar's approved bid covers General Works + Demo combined ($57,100). Column C shows Fabiano's General Works line on its own.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Negotiation target from Inputs. Fabiano's quote is in column C.</t>
         </r>
       </text>
     </comment>
@@ -148,7 +160,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="C33" authorId="0">
+    <comment ref="C38" authorId="0">
       <text>
         <r>
           <rPr>
@@ -165,7 +177,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="277">
   <si>
     <t xml:space="preserve">439 Manning Ave: Construction Plan</t>
   </si>
@@ -218,7 +230,7 @@
     <t xml:space="preserve">Pino (La Vecchia Designs)</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS (as of Oct 20, 2026)</t>
+    <t xml:space="preserve">STATUS (as of Oct 22, 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -260,7 +272,7 @@
     <t xml:space="preserve">Tendering</t>
   </si>
   <si>
-    <t xml:space="preserve">Bids in for most divisions; Fabiano, Doctor Demo and New Age still pending. Deadline Thu Oct 22, 7 PM (David).</t>
+    <t xml:space="preserve">Fabiano in Oct 22 ($37,900). Still pending: Doctor Demo, New Age and JB Contracting (framing), Honest Roofing, Milan Insulation. Deadline Thu Oct 22, 7 PM (David).</t>
   </si>
   <si>
     <t xml:space="preserve">Construction schedule</t>
@@ -317,7 +329,7 @@
     <t xml:space="preserve">1.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fabiano's General Works price decides the margin. Confirm it includes demo, licensed electrical + ESA, and drywall/insulation/trim materials.</t>
+    <t xml:space="preserve">Fabiano quoted $37,900: General Works $30,500 + demo $7,400. The plan assumes General Works negotiated to $25,000. At his full quote the margin drops about 5 points.</t>
   </si>
   <si>
     <t xml:space="preserve">2.</t>
@@ -425,7 +437,7 @@
     <t xml:space="preserve">Demolition: rear roof removal + temporary weather protection</t>
   </si>
   <si>
-    <t xml:space="preserve">Fabiano / demo contractor</t>
+    <t xml:space="preserve">FV Renovations (Fabiano)</t>
   </si>
   <si>
     <t xml:space="preserve">Framing: floor system, walls, flat roof, beams, ridge raise</t>
@@ -443,7 +455,7 @@
     <t xml:space="preserve">Flat roofing, parapet flashing, skylight</t>
   </si>
   <si>
-    <t xml:space="preserve">Safety Roofing</t>
+    <t xml:space="preserve">Prime Seal (roof) / skylight installer</t>
   </si>
   <si>
     <t xml:space="preserve">Window install (client-supplied units)</t>
@@ -455,6 +467,9 @@
     <t xml:space="preserve">Siding / cladding + flashing</t>
   </si>
   <si>
+    <t xml:space="preserve">Baz Aluminum</t>
+  </si>
+  <si>
     <t xml:space="preserve">HVAC rough-in + electrical rough-in</t>
   </si>
   <si>
@@ -764,7 +779,7 @@
     <t xml:space="preserve">Site Services has no quote yet; the $11,500 budget is carried at cost.</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm with Fabiano: demo as a separate line, licensed electrician + ESA included, and materials (drywall, insulation, trim) included.</t>
+    <t xml:space="preserve">Fabiano's General Works line includes licensed electrical + ESA, batts, vapour barrier, drywall, MDF trim and paint. Hardwood, doors and hardware are client-supplied (install only).</t>
   </si>
   <si>
     <t xml:space="preserve">439 Manning Ave: Bid Leveling Inputs</t>
@@ -794,34 +809,34 @@
     <t xml:space="preserve">Tendering SOP: cost target = contract sell / 1.35.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fabiano General Works price (estimate)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raff's estimate, Oct 20. Replace with the real number when it comes in.</t>
+    <t xml:space="preserve">Fabiano General Works price (negotiated target)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raff's negotiation target, Oct 22. Fabiano quoted $30,500 for General Works (JobTread bid #15). Change to the agreed number.</t>
   </si>
   <si>
     <t xml:space="preserve">Does Fabiano's price include demolition? (Yes/No)</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The work order asks for demo as a separate line. If No, the demo cost below gets added.</t>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabiano priced demo as a separate line ($7,400), per the work order.</t>
   </si>
   <si>
     <t xml:space="preserve">Demolition cost if separate</t>
   </si>
   <si>
-    <t xml:space="preserve">Internal demo budget (P7D). Replace with Fabiano's or Doctor Demo's price.</t>
+    <t xml:space="preserve">Fabiano demo line, JobTread bid #15 (Oct 22). Doctor Demo still pending.</t>
   </si>
   <si>
     <t xml:space="preserve">Roof + siding option (Split / Safety)</t>
   </si>
   <si>
-    <t xml:space="preserve">Safety</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Split = Alps roof + Baz siding. Safety = Safety Roofing combo (siding, flat roof and skylight).</t>
+    <t xml:space="preserve">Split</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split = lowest flat roof bid + lowest siding bid (now Prime Seal $5,900 + Baz $7,900). Safety = Safety Roofing combo $20,580 (siding, flat roof and skylight).</t>
   </si>
   <si>
     <t xml:space="preserve">Construction contingency (% of cost)</t>
@@ -833,7 +848,7 @@
     <t xml:space="preserve">Tender Package P2 provisional / change order risk.</t>
   </si>
   <si>
-    <t xml:space="preserve">All Manning Bid Requests (from JobTread, Oct 20, 2026)</t>
+    <t xml:space="preserve">All Manning Bid Requests (from JobTread, Oct 22, 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Amounts are the cost entered on each JobTread bid request. HST treatment not confirmed. To add a bid, insert a row above the last one and copy column E down.</t>
@@ -860,18 +875,18 @@
     <t xml:space="preserve">Approved</t>
   </si>
   <si>
-    <t xml:space="preserve">FV Renovations (Fabiano)</t>
+    <t xml:space="preserve">General Works (excl. demo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demolition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doctor Demo (Roman)</t>
   </si>
   <si>
     <t xml:space="preserve">Pending</t>
   </si>
   <si>
-    <t xml:space="preserve">Demolition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doctor Demo (Roman)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bradley Demolition</t>
   </si>
   <si>
@@ -893,6 +908,9 @@
     <t xml:space="preserve">Bogdan</t>
   </si>
   <si>
+    <t xml:space="preserve">JB Contracting (Jim)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lumber</t>
   </si>
   <si>
@@ -914,12 +932,15 @@
     <t xml:space="preserve">Ebi</t>
   </si>
   <si>
+    <t xml:space="preserve">Prime Seal Roofing Systems (Ellery)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Honest Roofing</t>
+  </si>
+  <si>
     <t xml:space="preserve">Siding</t>
   </si>
   <si>
-    <t xml:space="preserve">Baz Aluminum</t>
-  </si>
-  <si>
     <t xml:space="preserve">SM Cladding (Milos)</t>
   </si>
   <si>
@@ -945,6 +966,9 @@
   </si>
   <si>
     <t xml:space="preserve">FoamIt (Nadia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Milan Insulation (Andy Cruz)</t>
   </si>
   <si>
     <t xml:space="preserve">Windows (client-paid)</t>
@@ -1837,7 +1861,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>30</v>
       </c>
@@ -1934,7 +1958,7 @@
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">Leveling!$E$20</f>
-        <v>122296.69</v>
+        <v>115516.69</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -1946,7 +1970,7 @@
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">Leveling!$F$20</f>
-        <v>85196.69</v>
+        <v>90816.69</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -1958,7 +1982,7 @@
       </c>
       <c r="B28" s="9" t="n">
         <f aca="false">Leveling!$E$23</f>
-        <v>-0.0721196633646007</v>
+        <v>-0.0126824756728325</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -1970,7 +1994,7 @@
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">Leveling!$F$23</f>
-        <v>0.253119225037258</v>
+        <v>0.203851231699833</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -1982,7 +2006,7 @@
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">Leveling!$F$32</f>
-        <v>0.134598413255019</v>
+        <v>0.0804036205838521</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -2404,7 +2428,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="n">
         <v>5</v>
       </c>
@@ -2460,7 +2484,7 @@
         <v>95</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>2</v>
@@ -2481,10 +2505,10 @@
         <v>8</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>1.5</v>
@@ -2498,10 +2522,10 @@
         <v>46463</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2509,10 +2533,10 @@
         <v>9</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>1</v>
@@ -2526,7 +2550,7 @@
         <v>46470</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H19" s="16"/>
     </row>
@@ -2535,10 +2559,10 @@
         <v>10</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>2</v>
@@ -2553,7 +2577,7 @@
       </c>
       <c r="G20" s="16"/>
       <c r="H20" s="16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2561,10 +2585,10 @@
         <v>11</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>1</v>
@@ -2585,10 +2609,10 @@
         <v>12</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>1.5</v>
@@ -2603,7 +2627,7 @@
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2611,10 +2635,10 @@
         <v>13</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D23" s="12" t="n">
         <v>1</v>
@@ -2628,7 +2652,7 @@
         <v>46509</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H23" s="16"/>
     </row>
@@ -2637,10 +2661,10 @@
         <v>14</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D24" s="12" t="n">
         <v>1</v>
@@ -2654,10 +2678,10 @@
         <v>46516</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H24" s="16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2672,7 +2696,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -2713,7 +2737,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2726,7 +2750,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2756,7 +2780,7 @@
         <v>123030.16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -2767,7 +2791,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>0.13</v>
@@ -2782,7 +2806,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">B4-Inputs!$B$5</f>
@@ -2809,36 +2833,36 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F8" s="15" t="s">
         <v>20</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B9" s="23" t="n">
         <v>0.05</v>
@@ -2856,7 +2880,7 @@
         <v>6951.20404</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G9" s="24" t="n">
         <f aca="false">IF(F9="Paid",E9,0)</f>
@@ -2867,12 +2891,12 @@
         <v>0</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B10" s="23" t="n">
         <v>0.1</v>
@@ -2890,7 +2914,7 @@
         <v>13902.40808</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">IF(F10="Paid",E10,0)</f>
@@ -2901,12 +2925,12 @@
         <v>13902.40808</v>
       </c>
       <c r="I10" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B11" s="23" t="n">
         <v>0.15</v>
@@ -2924,7 +2948,7 @@
         <v>20853.61212</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G11" s="24" t="n">
         <f aca="false">IF(F11="Paid",E11,0)</f>
@@ -2941,7 +2965,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B12" s="23" t="n">
         <v>0.3</v>
@@ -2959,7 +2983,7 @@
         <v>41707.22424</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G12" s="24" t="n">
         <f aca="false">IF(F12="Paid",E12,0)</f>
@@ -2976,7 +3000,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B13" s="23" t="n">
         <v>0.15</v>
@@ -2994,7 +3018,7 @@
         <v>20853.61212</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G13" s="24" t="n">
         <f aca="false">IF(F13="Paid",E13,0)</f>
@@ -3011,7 +3035,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B14" s="23" t="n">
         <v>0.1</v>
@@ -3029,7 +3053,7 @@
         <v>13902.40808</v>
       </c>
       <c r="F14" s="25" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G14" s="24" t="n">
         <f aca="false">IF(F14="Paid",E14,0)</f>
@@ -3046,7 +3070,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B15" s="23" t="n">
         <v>0.1</v>
@@ -3064,7 +3088,7 @@
         <v>13902.40808</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G15" s="24" t="n">
         <f aca="false">IF(F15="Paid",E15,0)</f>
@@ -3081,7 +3105,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B16" s="23" t="n">
         <v>0.05</v>
@@ -3099,7 +3123,7 @@
         <v>6951.20404</v>
       </c>
       <c r="F16" s="25" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G16" s="24" t="n">
         <f aca="false">IF(F16="Paid",E16,0)</f>
@@ -3116,7 +3140,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="27" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B17" s="28" t="n">
         <f aca="false">SUM(B9:B16)</f>
@@ -3161,7 +3185,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -3202,7 +3226,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3216,7 +3240,7 @@
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="str">
         <f aca="false">"Scenario: Fabiano at "&amp;TEXT(Inputs!$B$7,"$#,##0")&amp;IF(Inputs!$B$8="Yes"," incl. demo"," + demo "&amp;TEXT(Inputs!$B$9,"$#,##0"))&amp;" | Roof/siding: "&amp;Inputs!$B$10</f>
-        <v>Scenario: Fabiano at $20,000 incl. demo | Roof/siding: Safety</v>
+        <v>Scenario: Fabiano at $25,000 + demo $7,400 | Roof/siding: Split</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3240,62 +3264,62 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E4" s="30" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F4" s="30" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G4" s="30" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H4" s="30" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I4" s="30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B5" s="31" t="n">
         <v>30041</v>
       </c>
       <c r="C5" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"General Works + Demo",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
-        <v>57100</v>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"General Works (excl. demo)",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <v>30500</v>
       </c>
       <c r="D5" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("General Works + Demo|"&amp;ROUND(C5,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
-        <v>Renomar Inc (Olimpiu)</v>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("General Works (excl. demo)|"&amp;ROUND(C5,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <v>FV Renovations (Fabiano)</v>
       </c>
       <c r="E5" s="24" t="n">
-        <f aca="false">C5</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"General Works + Demo",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>57100</v>
       </c>
       <c r="F5" s="24" t="n">
         <f aca="false">Inputs!$B$7</f>
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="G5" s="24" t="n">
         <f aca="false">F5-B5</f>
-        <v>-10041</v>
+        <v>-5041</v>
       </c>
       <c r="H5" s="33" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$34,"General Works + Demo",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"General Works (excl. demo)",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="I5" s="25" t="n">
@@ -3304,33 +3328,33 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B6" s="31" t="n">
         <v>6290</v>
       </c>
       <c r="C6" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Demolition",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
-        <v>0</v>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Demolition",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <v>7400</v>
       </c>
       <c r="D6" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Demolition|"&amp;ROUND(C6,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
-        <v>No price yet</v>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Demolition|"&amp;ROUND(C6,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <v>FV Renovations (Fabiano)</v>
       </c>
       <c r="E6" s="24" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="24" t="n">
         <f aca="false">IF(Inputs!$B$8="Yes",0,Inputs!$B$9)</f>
-        <v>0</v>
+        <v>7400</v>
       </c>
       <c r="G6" s="24" t="n">
         <f aca="false">F6-B6</f>
-        <v>-6290</v>
+        <v>1110</v>
       </c>
       <c r="H6" s="33" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$34,"Demolition",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Demolition",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <v>1</v>
       </c>
       <c r="I6" s="25" t="n">
         <v>3</v>
@@ -3338,17 +3362,17 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B7" s="31" t="n">
         <v>23128</v>
       </c>
       <c r="C7" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Framing",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Framing",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>14000</v>
       </c>
       <c r="D7" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Framing|"&amp;ROUND(C7,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Framing|"&amp;ROUND(C7,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>Aryan</v>
       </c>
       <c r="E7" s="24" t="n">
@@ -3364,7 +3388,7 @@
         <v>-9128</v>
       </c>
       <c r="H7" s="33" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$34,"Framing",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Framing",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="I7" s="25" t="n">
@@ -3373,17 +3397,17 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B8" s="31" t="n">
         <v>4900</v>
       </c>
       <c r="C8" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Lumber",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Lumber",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>6386.19</v>
       </c>
       <c r="D8" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Lumber|"&amp;ROUND(C8,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Lumber|"&amp;ROUND(C8,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>RONA (Jonathan)</v>
       </c>
       <c r="E8" s="24" t="n">
@@ -3399,7 +3423,7 @@
         <v>1486.19</v>
       </c>
       <c r="H8" s="33" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$34,"Lumber",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Lumber",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>3</v>
       </c>
       <c r="I8" s="25" t="n">
@@ -3408,34 +3432,34 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B9" s="31" t="n">
         <v>8010</v>
       </c>
       <c r="C9" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Flat Roofing",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
-        <v>15700</v>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Flat Roofing",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <v>5900</v>
       </c>
       <c r="D9" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Flat Roofing|"&amp;ROUND(C9,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
-        <v>Alps Roofing</v>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Flat Roofing|"&amp;ROUND(C9,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <v>Prime Seal Roofing Systems (Ellery)</v>
       </c>
       <c r="E9" s="24" t="n">
         <f aca="false">IF(Inputs!$B$10="Split",C9,0)</f>
-        <v>0</v>
+        <v>5900</v>
       </c>
       <c r="F9" s="24" t="n">
         <f aca="false">E9</f>
-        <v>0</v>
+        <v>5900</v>
       </c>
       <c r="G9" s="24" t="n">
         <f aca="false">IF(Inputs!$B$10="Split",F9-B9,0)</f>
-        <v>0</v>
+        <v>-2110</v>
       </c>
       <c r="H9" s="33" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$34,"Flat Roofing",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Flat Roofing",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <v>2</v>
       </c>
       <c r="I9" s="25" t="n">
         <v>3</v>
@@ -3443,33 +3467,33 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B10" s="31" t="n">
         <v>17750</v>
       </c>
       <c r="C10" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Siding",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Siding",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>7900</v>
       </c>
       <c r="D10" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Siding|"&amp;ROUND(C10,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Siding|"&amp;ROUND(C10,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>Baz Aluminum</v>
       </c>
       <c r="E10" s="24" t="n">
         <f aca="false">IF(Inputs!$B$10="Split",C10,0)</f>
-        <v>0</v>
+        <v>7900</v>
       </c>
       <c r="F10" s="24" t="n">
         <f aca="false">E10</f>
-        <v>0</v>
+        <v>7900</v>
       </c>
       <c r="G10" s="24" t="n">
         <f aca="false">IF(Inputs!$B$10="Split",F10-B10,0)</f>
-        <v>0</v>
+        <v>-9850</v>
       </c>
       <c r="H10" s="33" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$34,"Siding",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Siding",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="I10" s="25" t="n">
@@ -3478,33 +3502,33 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B11" s="31" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Roof + Siding + Skylight Combo",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Roof + Siding + Skylight Combo",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>20580</v>
       </c>
       <c r="D11" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Roof + Siding + Skylight Combo|"&amp;ROUND(C11,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Roof + Siding + Skylight Combo|"&amp;ROUND(C11,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>Safety Roofing (Elvis)</v>
       </c>
       <c r="E11" s="24" t="n">
         <f aca="false">IF(Inputs!$B$10="Split",0,C11)</f>
-        <v>20580</v>
+        <v>0</v>
       </c>
       <c r="F11" s="24" t="n">
         <f aca="false">E11</f>
-        <v>20580</v>
+        <v>0</v>
       </c>
       <c r="G11" s="24" t="n">
         <f aca="false">IF(Inputs!$B$10="Split",0,F11-(B9+B10))</f>
-        <v>-5180</v>
+        <v>0</v>
       </c>
       <c r="H11" s="33" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$34,"Roof + Siding + Skylight Combo",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Roof + Siding + Skylight Combo",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="I11" s="25" t="n">
@@ -3513,17 +3537,17 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B12" s="31" t="n">
         <v>6750</v>
       </c>
       <c r="C12" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"HVAC",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"HVAC",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>9370</v>
       </c>
       <c r="D12" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("HVAC|"&amp;ROUND(C12,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("HVAC|"&amp;ROUND(C12,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>Ideal Heating (Leena)</v>
       </c>
       <c r="E12" s="24" t="n">
@@ -3539,7 +3563,7 @@
         <v>2620</v>
       </c>
       <c r="H12" s="33" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$34,"HVAC",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"HVAC",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>2</v>
       </c>
       <c r="I12" s="25" t="n">
@@ -3548,17 +3572,17 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B13" s="31" t="n">
         <v>3430</v>
       </c>
       <c r="C13" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Spray Foam",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Spray Foam",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>3360.5</v>
       </c>
       <c r="D13" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Spray Foam|"&amp;ROUND(C13,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Spray Foam|"&amp;ROUND(C13,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>FoamIt (Nadia)</v>
       </c>
       <c r="E13" s="24" t="n">
@@ -3574,7 +3598,7 @@
         <v>-69.5</v>
       </c>
       <c r="H13" s="33" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$34,"Spray Foam",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Spray Foam",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="I13" s="25" t="n">
@@ -3583,7 +3607,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B14" s="31" t="n">
         <v>11500</v>
@@ -3592,7 +3616,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E14" s="24" t="n">
         <f aca="false">B14</f>
@@ -3615,7 +3639,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B15" s="29" t="n">
         <f aca="false">SUM(B5:B14)</f>
@@ -3625,15 +3649,15 @@
       <c r="D15" s="27"/>
       <c r="E15" s="29" t="n">
         <f aca="false">SUM(E5:E14)</f>
-        <v>122296.69</v>
+        <v>115516.69</v>
       </c>
       <c r="F15" s="29" t="n">
         <f aca="false">SUM(F5:F14)</f>
-        <v>85196.69</v>
+        <v>90816.69</v>
       </c>
       <c r="G15" s="29" t="n">
         <f aca="false">SUM(G5:G14)</f>
-        <v>-26602.31</v>
+        <v>-20982.31</v>
       </c>
       <c r="H15" s="27"/>
       <c r="I15" s="27"/>
@@ -3651,16 +3675,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
       <c r="E17" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -3668,7 +3692,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -3687,7 +3711,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -3706,18 +3730,18 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="34" t="n">
         <f aca="false">E15</f>
-        <v>122296.69</v>
+        <v>115516.69</v>
       </c>
       <c r="F20" s="34" t="n">
         <f aca="false">F15</f>
-        <v>85196.69</v>
+        <v>90816.69</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -3725,18 +3749,18 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="35" t="n">
         <f aca="false">E20-E19</f>
-        <v>37800.3937037037</v>
+        <v>31020.3937037037</v>
       </c>
       <c r="F21" s="35" t="n">
         <f aca="false">F20-F19</f>
-        <v>700.39370370371</v>
+        <v>6320.39370370371</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -3744,18 +3768,18 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="34" t="n">
         <f aca="false">E18-E20</f>
-        <v>-8226.69</v>
+        <v>-1446.69</v>
       </c>
       <c r="F22" s="34" t="n">
         <f aca="false">F18-F20</f>
-        <v>28873.31</v>
+        <v>23253.31</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -3763,18 +3787,18 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="36" t="n">
         <f aca="false">IF(E18=0,0,E22/E18)</f>
-        <v>-0.0721196633646007</v>
+        <v>-0.0126824756728325</v>
       </c>
       <c r="F23" s="36" t="n">
         <f aca="false">IF(F18=0,0,F22/F18)</f>
-        <v>0.253119225037258</v>
+        <v>0.203851231699833</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
@@ -3782,18 +3806,18 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="36" t="n">
         <f aca="false">IF(E20=0,0,E22/E20)</f>
-        <v>-0.0672682964682037</v>
+        <v>-0.012523644851666</v>
       </c>
       <c r="F24" s="36" t="n">
         <f aca="false">IF(F20=0,0,F22/F20)</f>
-        <v>0.338901781278122</v>
+        <v>0.256046658384048</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -3801,7 +3825,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -3831,7 +3855,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -3844,18 +3868,18 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="34" t="n">
         <f aca="false">E20*Inputs!$B$11</f>
-        <v>12229.669</v>
+        <v>11551.669</v>
       </c>
       <c r="F28" s="34" t="n">
         <f aca="false">F20*Inputs!$B$11</f>
-        <v>8519.669</v>
+        <v>9081.669</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -3863,7 +3887,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -3882,18 +3906,18 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="35" t="n">
         <f aca="false">E20+E28+E29</f>
-        <v>139526.359</v>
+        <v>132068.359</v>
       </c>
       <c r="F30" s="35" t="n">
         <f aca="false">F20+F28+F29</f>
-        <v>98716.359</v>
+        <v>104898.359</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -3901,18 +3925,18 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="34" t="n">
         <f aca="false">E18-E30</f>
-        <v>-25456.359</v>
+        <v>-17998.359</v>
       </c>
       <c r="F31" s="34" t="n">
         <f aca="false">F18-F30</f>
-        <v>15353.641</v>
+        <v>9171.641</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -3920,18 +3944,18 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="36" t="n">
         <f aca="false">IF(E18=0,0,E31/E18)</f>
-        <v>-0.223164363987026</v>
+        <v>-0.15778345752608</v>
       </c>
       <c r="F32" s="36" t="n">
         <f aca="false">IF(F18=0,0,F31/F18)</f>
-        <v>0.134598413255019</v>
+        <v>0.0804036205838521</v>
       </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
@@ -3950,7 +3974,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="37" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -3963,42 +3987,42 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B36" s="31" t="n">
         <v>36400</v>
       </c>
       <c r="C36" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Add-on: Brick Veneer",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Add-on: Brick Veneer",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>31200</v>
       </c>
       <c r="D36" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Add-on: Brick Veneer|"&amp;ROUND(C36,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Add-on: Brick Veneer|"&amp;ROUND(C36,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>Amoroso Construction</v>
       </c>
       <c r="E36" s="31" t="n">
@@ -4017,17 +4041,17 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B37" s="31" t="n">
         <v>3960</v>
       </c>
       <c r="C37" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Add-on: Interior Brick",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Add-on: Interior Brick",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>10800</v>
       </c>
       <c r="D37" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Add-on: Interior Brick|"&amp;ROUND(C37,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Add-on: Interior Brick|"&amp;ROUND(C37,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>Amoroso Construction</v>
       </c>
       <c r="E37" s="31" t="n">
@@ -4046,17 +4070,17 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B38" s="31" t="n">
         <v>4600</v>
       </c>
       <c r="C38" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Add-on: Skylight",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Add-on: Skylight",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>3300</v>
       </c>
       <c r="D38" s="32" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Add-on: Skylight|"&amp;ROUND(C38,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Add-on: Skylight|"&amp;ROUND(C38,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>Skylight Services Ltd</v>
       </c>
       <c r="E38" s="31" t="n">
@@ -4086,17 +4110,17 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B40" s="20" t="n">
         <v>8470</v>
       </c>
       <c r="C40" s="38" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$34,'All Bids'!$A$5:$A$34,"Windows (client-paid)",'All Bids'!$C$5:$C$34,"Approved",'All Bids'!$D$5:$D$34,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Windows (client-paid)",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
         <v>7850</v>
       </c>
       <c r="D40" s="39" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$34,MATCH("Windows (client-paid)|"&amp;ROUND(C40,2),'All Bids'!$E$5:$E$34,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Windows (client-paid)|"&amp;ROUND(C40,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
         <v>JS Windows and Doors</v>
       </c>
       <c r="E40" s="2"/>
@@ -4107,14 +4131,14 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B41" s="20" t="n">
         <v>7549</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
@@ -4135,7 +4159,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -4148,7 +4172,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="19" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -4161,7 +4185,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="19" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -4174,7 +4198,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="19" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -4187,7 +4211,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="19" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -4200,7 +4224,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="19" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -4213,7 +4237,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="19" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -4226,7 +4250,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="19" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -4290,14 +4314,14 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4309,101 +4333,101 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="40" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B5" s="41" t="n">
         <v>114070</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="40" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B6" s="42" t="n">
         <v>0.35</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="40" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B7" s="41" t="n">
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="40" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="40" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B9" s="41" t="n">
-        <v>6290</v>
+        <v>7400</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="40" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="40" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B11" s="42" t="n">
         <v>0.1</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="40" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B12" s="41" t="n">
         <v>5000</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -4432,7 +4456,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="32"/>
@@ -4444,7 +4468,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4454,7 +4478,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4472,33 +4496,33 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>20</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B5" s="43" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>57100</v>
@@ -4513,20 +4537,20 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B6" s="43" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="43" t="s">
         <v>231</v>
       </c>
-      <c r="C6" s="43" t="s">
-        <v>232</v>
-      </c>
       <c r="D6" s="31" t="n">
-        <v>0</v>
+        <v>30500</v>
       </c>
       <c r="E6" s="16" t="str">
         <f aca="false">IF(AND(C6="Approved",D6&gt;0),A6&amp;"|"&amp;ROUND(D6,2),"")</f>
-        <v/>
+        <v>General Works (excl. demo)|30500</v>
       </c>
       <c r="F6" s="25" t="n">
         <v>15</v>
@@ -4537,20 +4561,20 @@
         <v>233</v>
       </c>
       <c r="B7" s="43" t="s">
-        <v>234</v>
+        <v>86</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D7" s="31" t="n">
-        <v>0</v>
+        <v>7400</v>
       </c>
       <c r="E7" s="16" t="str">
         <f aca="false">IF(AND(C7="Approved",D7&gt;0),A7&amp;"|"&amp;ROUND(D7,2),"")</f>
-        <v/>
+        <v>Demolition|7400</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4558,10 +4582,10 @@
         <v>233</v>
       </c>
       <c r="B8" s="43" t="s">
+        <v>234</v>
+      </c>
+      <c r="C8" s="43" t="s">
         <v>235</v>
-      </c>
-      <c r="C8" s="43" t="s">
-        <v>236</v>
       </c>
       <c r="D8" s="31" t="n">
         <v>0</v>
@@ -4571,7 +4595,7 @@
         <v/>
       </c>
       <c r="F8" s="25" t="n">
-        <v>41</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4579,10 +4603,10 @@
         <v>233</v>
       </c>
       <c r="B9" s="43" t="s">
+        <v>236</v>
+      </c>
+      <c r="C9" s="43" t="s">
         <v>237</v>
-      </c>
-      <c r="C9" s="43" t="s">
-        <v>236</v>
       </c>
       <c r="D9" s="31" t="n">
         <v>0</v>
@@ -4592,60 +4616,60 @@
         <v/>
       </c>
       <c r="F9" s="25" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="43" t="s">
+        <v>233</v>
+      </c>
+      <c r="B10" s="43" t="s">
         <v>238</v>
       </c>
-      <c r="B10" s="43" t="s">
-        <v>239</v>
-      </c>
       <c r="C10" s="43" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D10" s="31" t="n">
-        <v>14000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="16" t="str">
         <f aca="false">IF(AND(C10="Approved",D10&gt;0),A10&amp;"|"&amp;ROUND(D10,2),"")</f>
-        <v>Framing|14000</v>
+        <v/>
       </c>
       <c r="F10" s="25" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="43" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B11" s="43" t="s">
         <v>240</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D11" s="31" t="n">
-        <v>0</v>
+        <v>14000</v>
       </c>
       <c r="E11" s="16" t="str">
         <f aca="false">IF(AND(C11="Approved",D11&gt;0),A11&amp;"|"&amp;ROUND(D11,2),"")</f>
-        <v/>
+        <v>Framing|14000</v>
       </c>
       <c r="F11" s="25" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="43" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B12" s="43" t="s">
         <v>241</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D12" s="31" t="n">
         <v>0</v>
@@ -4655,165 +4679,165 @@
         <v/>
       </c>
       <c r="F12" s="25" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="43" t="s">
+        <v>239</v>
+      </c>
+      <c r="B13" s="43" t="s">
         <v>242</v>
       </c>
-      <c r="B13" s="43" t="s">
-        <v>243</v>
-      </c>
       <c r="C13" s="43" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D13" s="31" t="n">
-        <v>6386.19</v>
+        <v>0</v>
       </c>
       <c r="E13" s="16" t="str">
         <f aca="false">IF(AND(C13="Approved",D13&gt;0),A13&amp;"|"&amp;ROUND(D13,2),"")</f>
-        <v>Lumber|6386.19</v>
+        <v/>
       </c>
       <c r="F13" s="25" t="n">
-        <v>43</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="43" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B14" s="43" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="D14" s="31" t="n">
-        <v>7040</v>
+        <v>0</v>
       </c>
       <c r="E14" s="16" t="str">
         <f aca="false">IF(AND(C14="Approved",D14&gt;0),A14&amp;"|"&amp;ROUND(D14,2),"")</f>
-        <v>Lumber|7040</v>
+        <v/>
       </c>
       <c r="F14" s="25" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="43" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B15" s="43" t="s">
         <v>245</v>
       </c>
       <c r="C15" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D15" s="31" t="n">
-        <v>7208.9</v>
+        <v>6386.19</v>
       </c>
       <c r="E15" s="16" t="str">
         <f aca="false">IF(AND(C15="Approved",D15&gt;0),A15&amp;"|"&amp;ROUND(D15,2),"")</f>
-        <v>Lumber|7208.9</v>
+        <v>Lumber|6386.19</v>
       </c>
       <c r="F15" s="25" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="43" t="s">
-        <v>157</v>
+        <v>244</v>
       </c>
       <c r="B16" s="43" t="s">
         <v>246</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D16" s="31" t="n">
-        <v>15700</v>
+        <v>7040</v>
       </c>
       <c r="E16" s="16" t="str">
         <f aca="false">IF(AND(C16="Approved",D16&gt;0),A16&amp;"|"&amp;ROUND(D16,2),"")</f>
-        <v>Flat Roofing|15700</v>
+        <v>Lumber|7040</v>
       </c>
       <c r="F16" s="25" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="43" t="s">
-        <v>157</v>
+        <v>244</v>
       </c>
       <c r="B17" s="43" t="s">
         <v>247</v>
       </c>
       <c r="C17" s="43" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="D17" s="31" t="n">
-        <v>0</v>
+        <v>7208.9</v>
       </c>
       <c r="E17" s="16" t="str">
         <f aca="false">IF(AND(C17="Approved",D17&gt;0),A17&amp;"|"&amp;ROUND(D17,2),"")</f>
-        <v/>
+        <v>Lumber|7208.9</v>
       </c>
       <c r="F17" s="25" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="43" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B18" s="43" t="s">
         <v>248</v>
       </c>
       <c r="C18" s="43" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="D18" s="31" t="n">
-        <v>0</v>
+        <v>15700</v>
       </c>
       <c r="E18" s="16" t="str">
         <f aca="false">IF(AND(C18="Approved",D18&gt;0),A18&amp;"|"&amp;ROUND(D18,2),"")</f>
-        <v/>
+        <v>Flat Roofing|15700</v>
       </c>
       <c r="F18" s="25" t="n">
-        <v>33</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="43" t="s">
+        <v>158</v>
+      </c>
+      <c r="B19" s="43" t="s">
         <v>249</v>
       </c>
-      <c r="B19" s="43" t="s">
-        <v>250</v>
-      </c>
       <c r="C19" s="43" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D19" s="31" t="n">
-        <v>7900</v>
+        <v>0</v>
       </c>
       <c r="E19" s="16" t="str">
         <f aca="false">IF(AND(C19="Approved",D19&gt;0),A19&amp;"|"&amp;ROUND(D19,2),"")</f>
-        <v>Siding|7900</v>
+        <v/>
       </c>
       <c r="F19" s="25" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="43" t="s">
-        <v>249</v>
+        <v>158</v>
       </c>
       <c r="B20" s="43" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C20" s="43" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D20" s="31" t="n">
         <v>0</v>
@@ -4823,81 +4847,81 @@
         <v/>
       </c>
       <c r="F20" s="25" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="43" t="s">
-        <v>252</v>
+        <v>158</v>
       </c>
       <c r="B21" s="43" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C21" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D21" s="31" t="n">
-        <v>20580</v>
+        <v>5900</v>
       </c>
       <c r="E21" s="16" t="str">
         <f aca="false">IF(AND(C21="Approved",D21&gt;0),A21&amp;"|"&amp;ROUND(D21,2),"")</f>
-        <v>Roof + Siding + Skylight Combo|20580</v>
+        <v>Flat Roofing|5900</v>
       </c>
       <c r="F21" s="25" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="43" t="s">
-        <v>254</v>
+        <v>158</v>
       </c>
       <c r="B22" s="43" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C22" s="43" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="D22" s="31" t="n">
-        <v>9370</v>
+        <v>0</v>
       </c>
       <c r="E22" s="16" t="str">
         <f aca="false">IF(AND(C22="Approved",D22&gt;0),A22&amp;"|"&amp;ROUND(D22,2),"")</f>
-        <v>HVAC|9370</v>
+        <v/>
       </c>
       <c r="F22" s="25" t="n">
-        <v>28</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="43" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B23" s="43" t="s">
-        <v>256</v>
+        <v>96</v>
       </c>
       <c r="C23" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D23" s="31" t="n">
-        <v>9950</v>
+        <v>7900</v>
       </c>
       <c r="E23" s="16" t="str">
         <f aca="false">IF(AND(C23="Approved",D23&gt;0),A23&amp;"|"&amp;ROUND(D23,2),"")</f>
-        <v>HVAC|9950</v>
+        <v>Siding|7900</v>
       </c>
       <c r="F23" s="25" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="43" t="s">
+        <v>253</v>
+      </c>
+      <c r="B24" s="43" t="s">
         <v>254</v>
       </c>
-      <c r="B24" s="43" t="s">
-        <v>257</v>
-      </c>
       <c r="C24" s="43" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D24" s="31" t="n">
         <v>0</v>
@@ -4907,216 +4931,321 @@
         <v/>
       </c>
       <c r="F24" s="25" t="n">
-        <v>27</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="43" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B25" s="43" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C25" s="43" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="D25" s="31" t="n">
-        <v>0</v>
+        <v>20580</v>
       </c>
       <c r="E25" s="16" t="str">
         <f aca="false">IF(AND(C25="Approved",D25&gt;0),A25&amp;"|"&amp;ROUND(D25,2),"")</f>
-        <v/>
+        <v>Roof + Siding + Skylight Combo|20580</v>
       </c>
       <c r="F25" s="25" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="43" t="s">
-        <v>161</v>
+        <v>257</v>
       </c>
       <c r="B26" s="43" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C26" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D26" s="31" t="n">
-        <v>3360.5</v>
+        <v>9370</v>
       </c>
       <c r="E26" s="16" t="str">
         <f aca="false">IF(AND(C26="Approved",D26&gt;0),A26&amp;"|"&amp;ROUND(D26,2),"")</f>
-        <v>Spray Foam|3360.5</v>
+        <v>HVAC|9370</v>
       </c>
       <c r="F26" s="25" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="43" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B27" s="43" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C27" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D27" s="31" t="n">
-        <v>7850</v>
+        <v>9950</v>
       </c>
       <c r="E27" s="16" t="str">
         <f aca="false">IF(AND(C27="Approved",D27&gt;0),A27&amp;"|"&amp;ROUND(D27,2),"")</f>
-        <v>Windows (client-paid)|7850</v>
+        <v>HVAC|9950</v>
       </c>
       <c r="F27" s="25" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="43" t="s">
+        <v>257</v>
+      </c>
+      <c r="B28" s="43" t="s">
         <v>260</v>
       </c>
-      <c r="B28" s="43" t="s">
-        <v>262</v>
-      </c>
       <c r="C28" s="43" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D28" s="31" t="n">
-        <v>8340</v>
+        <v>0</v>
       </c>
       <c r="E28" s="16" t="str">
         <f aca="false">IF(AND(C28="Approved",D28&gt;0),A28&amp;"|"&amp;ROUND(D28,2),"")</f>
-        <v>Windows (client-paid)|8340</v>
+        <v/>
       </c>
       <c r="F28" s="25" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="43" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B29" s="43" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C29" s="43" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D29" s="31" t="n">
-        <v>9646.02</v>
+        <v>0</v>
       </c>
       <c r="E29" s="16" t="str">
         <f aca="false">IF(AND(C29="Approved",D29&gt;0),A29&amp;"|"&amp;ROUND(D29,2),"")</f>
-        <v>Windows (client-paid)|9646.02</v>
+        <v/>
       </c>
       <c r="F29" s="25" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="43" t="s">
-        <v>264</v>
+        <v>162</v>
       </c>
       <c r="B30" s="43" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C30" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D30" s="31" t="n">
-        <v>31200</v>
+        <v>3360.5</v>
       </c>
       <c r="E30" s="16" t="str">
         <f aca="false">IF(AND(C30="Approved",D30&gt;0),A30&amp;"|"&amp;ROUND(D30,2),"")</f>
-        <v>Add-on: Brick Veneer|31200</v>
+        <v>Spray Foam|3360.5</v>
       </c>
       <c r="F30" s="25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="43" t="s">
-        <v>266</v>
+        <v>162</v>
       </c>
       <c r="B31" s="43" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C31" s="43" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="D31" s="31" t="n">
-        <v>10800</v>
+        <v>0</v>
       </c>
       <c r="E31" s="16" t="str">
         <f aca="false">IF(AND(C31="Approved",D31&gt;0),A31&amp;"|"&amp;ROUND(D31,2),"")</f>
-        <v>Add-on: Interior Brick|10800</v>
+        <v/>
       </c>
       <c r="F31" s="25" t="n">
-        <v>14</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="43" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B32" s="43" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C32" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D32" s="31" t="n">
-        <v>3300</v>
+        <v>7850</v>
       </c>
       <c r="E32" s="16" t="str">
         <f aca="false">IF(AND(C32="Approved",D32&gt;0),A32&amp;"|"&amp;ROUND(D32,2),"")</f>
-        <v>Add-on: Skylight|3300</v>
+        <v>Windows (client-paid)|7850</v>
       </c>
       <c r="F32" s="25" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="43" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B33" s="43" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C33" s="43" t="s">
-        <v>270</v>
+        <v>231</v>
       </c>
       <c r="D33" s="31" t="n">
-        <v>300</v>
+        <v>8340</v>
       </c>
       <c r="E33" s="16" t="str">
         <f aca="false">IF(AND(C33="Approved",D33&gt;0),A33&amp;"|"&amp;ROUND(D33,2),"")</f>
-        <v/>
+        <v>Windows (client-paid)|8340</v>
       </c>
       <c r="F33" s="25" t="n">
-        <v>26</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="43" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="B34" s="43" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="C34" s="43" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D34" s="31" t="n">
-        <v>1215</v>
+        <v>9646.02</v>
       </c>
       <c r="E34" s="16" t="str">
         <f aca="false">IF(AND(C34="Approved",D34&gt;0),A34&amp;"|"&amp;ROUND(D34,2),"")</f>
+        <v>Windows (client-paid)|9646.02</v>
+      </c>
+      <c r="F34" s="25" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="43" t="s">
+        <v>268</v>
+      </c>
+      <c r="B35" s="43" t="s">
+        <v>269</v>
+      </c>
+      <c r="C35" s="43" t="s">
+        <v>231</v>
+      </c>
+      <c r="D35" s="31" t="n">
+        <v>31200</v>
+      </c>
+      <c r="E35" s="16" t="str">
+        <f aca="false">IF(AND(C35="Approved",D35&gt;0),A35&amp;"|"&amp;ROUND(D35,2),"")</f>
+        <v>Add-on: Brick Veneer|31200</v>
+      </c>
+      <c r="F35" s="25" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="43" t="s">
+        <v>270</v>
+      </c>
+      <c r="B36" s="43" t="s">
+        <v>269</v>
+      </c>
+      <c r="C36" s="43" t="s">
+        <v>231</v>
+      </c>
+      <c r="D36" s="31" t="n">
+        <v>10800</v>
+      </c>
+      <c r="E36" s="16" t="str">
+        <f aca="false">IF(AND(C36="Approved",D36&gt;0),A36&amp;"|"&amp;ROUND(D36,2),"")</f>
+        <v>Add-on: Interior Brick|10800</v>
+      </c>
+      <c r="F36" s="25" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="B37" s="43" t="s">
+        <v>272</v>
+      </c>
+      <c r="C37" s="43" t="s">
+        <v>231</v>
+      </c>
+      <c r="D37" s="31" t="n">
+        <v>3300</v>
+      </c>
+      <c r="E37" s="16" t="str">
+        <f aca="false">IF(AND(C37="Approved",D37&gt;0),A37&amp;"|"&amp;ROUND(D37,2),"")</f>
+        <v>Add-on: Skylight|3300</v>
+      </c>
+      <c r="F37" s="25" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="B38" s="43" t="s">
+        <v>273</v>
+      </c>
+      <c r="C38" s="43" t="s">
+        <v>274</v>
+      </c>
+      <c r="D38" s="31" t="n">
+        <v>300</v>
+      </c>
+      <c r="E38" s="16" t="str">
+        <f aca="false">IF(AND(C38="Approved",D38&gt;0),A38&amp;"|"&amp;ROUND(D38,2),"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="25" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="43" t="s">
+        <v>275</v>
+      </c>
+      <c r="B39" s="43" t="s">
+        <v>276</v>
+      </c>
+      <c r="C39" s="43" t="s">
+        <v>231</v>
+      </c>
+      <c r="D39" s="31" t="n">
+        <v>1215</v>
+      </c>
+      <c r="E39" s="16" t="str">
+        <f aca="false">IF(AND(C39="Approved",D39&gt;0),A39&amp;"|"&amp;ROUND(D39,2),"")</f>
         <v>Hardwood Install (in GW scope)|1215</v>
       </c>
-      <c r="F34" s="25" t="n">
+      <c r="F39" s="25" t="n">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Manning plan: Leveling 2.0 negotiated targets, scope gap lines, new bids
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY6xq9eh2BK6Au4SE2w7Bc
</commit_message>
<xml_diff>
--- a/Manning_Construction_Plan.xlsx
+++ b/Manning_Construction_Plan.xlsx
@@ -161,7 +161,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="A21" authorId="0">
+    <comment ref="A23" authorId="0">
       <text>
         <r>
           <rPr>
@@ -181,11 +181,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Raff's carry. Fabiano's quote is $30,500 (JobTread bid #15, General Works line).</t>
+          <t xml:space="preserve">Fabiano bid #15: General Works $30,500 + Demolition $7,400.</t>
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="0">
+    <comment ref="E12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -193,11 +193,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Raff's estimate. Lowest framing bid received is Aryan at $14,000; New Age and JB Contracting still pending.</t>
+          <t xml:space="preserve">Stephenson's #66: scaffold $482 x 3 mo = $1,446; hoist $1,187 x 3 + $170 = $3,731; bins $350 x 2 x 4 mo = $2,800. United #64: toilet $150 x 3 + $550 = $1,000. Plus $1,500 boom-truck / roof-level deliveries.</t>
         </r>
       </text>
     </comment>
-    <comment ref="E11" authorId="0">
+    <comment ref="E13" authorId="0">
       <text>
         <r>
           <rPr>
@@ -205,7 +205,19 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">MiTech Quote #611 lists both options and adds them together ($9,950). Option 2 = $3,200 + $250 vent runs. Quote dated Apr 21, 2026, valid 30 days: re-confirm.</t>
+          <t xml:space="preserve">Tender Package budget: ridge raise framing $2,640 + re-shingle $960. No trade has priced it.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">PalmView allowance, not a quote.</t>
         </r>
       </text>
     </comment>
@@ -219,7 +231,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="C38" authorId="0">
+    <comment ref="C51" authorId="0">
       <text>
         <r>
           <rPr>
@@ -236,7 +248,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="346">
   <si>
     <t xml:space="preserve">439 Manning Ave: Construction Plan</t>
   </si>
@@ -289,7 +301,7 @@
     <t xml:space="preserve">Pino (La Vecchia Designs)</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS (as of Oct 22, 2026)</t>
+    <t xml:space="preserve">STATUS (as of Oct 25, 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -328,7 +340,7 @@
     <t xml:space="preserve">Tendering</t>
   </si>
   <si>
-    <t xml:space="preserve">Fabiano in Oct 22 ($37,900). Still pending: Doctor Demo, New Age and JB Contracting (framing), Honest Roofing, Milan Insulation. Deadline Thu Oct 22, 7 PM (David).</t>
+    <t xml:space="preserve">All key divisions priced. Negotiating to the Leveling 2.0 targets. Still pending: Doctor Demo, New Age, JB Contracting, Honest Roofing, Wallcent. Elvis (Safety Roofing) re-price due Mon Oct 26, 6 PM (David).</t>
   </si>
   <si>
     <t xml:space="preserve">In progress</t>
@@ -358,19 +370,19 @@
     <t xml:space="preserve">Cost target at 35% markup</t>
   </si>
   <si>
-    <t xml:space="preserve">Base cost: Leveling 2.0 (carried)</t>
+    <t xml:space="preserve">Base cost: required (negotiated)</t>
   </si>
   <si>
     <t xml:space="preserve">Base cost: at quoted prices</t>
   </si>
   <si>
-    <t xml:space="preserve">Margin: Leveling 2.0 (carried)</t>
+    <t xml:space="preserve">Margin: required (negotiated)</t>
   </si>
   <si>
     <t xml:space="preserve">Margin: at quoted prices</t>
   </si>
   <si>
-    <t xml:space="preserve">All-in margin, Leveling 2.0 (incl. contingency + provisional)</t>
+    <t xml:space="preserve">All-in margin, required (incl. contingency + provisional)</t>
   </si>
   <si>
     <t xml:space="preserve">Collected to date (incl. HST)</t>
@@ -385,13 +397,13 @@
     <t xml:space="preserve">1.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fabiano quoted $37,900: General Works $30,500 + demo $7,400. Leveling 2.0 carries General Works at $27,000 and framing at $10,000 (low bid $14,000). Both need to be locked in.</t>
+    <t xml:space="preserve">Negotiation targets (Leveling 2.0): Fabiano all-in $32,250 (quoted $37,900), Aryan $12,000 ($14,000), Baz $7,000 ($7,900), spray foam $3,200, RONA $6,500 (max $7,000), Prime Seal $6,000 with aluminum.</t>
   </si>
   <si>
     <t xml:space="preserve">2.</t>
   </si>
   <si>
-    <t xml:space="preserve">Brick veneer add-on: lowest bid $31,200 vs about $8,000 told to the client. Re-quote before Kyle, Nancy or neighbour Peter commit.</t>
+    <t xml:space="preserve">Add-ons re-priced: exterior brick veneer now $8,320 (Masonry Professionals), close to the ~$8,000 told to the client. Interior brick $5,850 vs ~$3,600 quoted.</t>
   </si>
   <si>
     <t xml:space="preserve">3.</t>
@@ -409,13 +421,13 @@
     <t xml:space="preserve">5.</t>
   </si>
   <si>
-    <t xml:space="preserve">Winter build: the roof is open from demo until the flat roof is on (about 4.5 weeks in Jan to Feb). Budget temporary heat and weather protection, or hold demo until the permit date is firm.</t>
+    <t xml:space="preserve">Winter build: roof open from demo until the flat roof is on (about 4 weeks, Jan to Feb). $1,500 winter protection allowance carried. Ridge raise ($3,600 allowance) still unpriced.</t>
   </si>
   <si>
     <t xml:space="preserve">6.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bedroom egress window and side-wall limiting distance to be confirmed with the designer before windows are ordered.</t>
+    <t xml:space="preserve">Window count mismatch: Aryan priced 6 openings, drawings show 4. Confirm with La Vecchia, plus bedroom egress and side-wall limiting distance.</t>
   </si>
   <si>
     <t xml:space="preserve">7.</t>
@@ -520,7 +532,7 @@
     <t xml:space="preserve">Framing: floor system, walls, flat roof, beams, ridge raise</t>
   </si>
   <si>
-    <t xml:space="preserve">Framer TBD + RONA lumber</t>
+    <t xml:space="preserve">Aryan + RONA lumber</t>
   </si>
   <si>
     <t xml:space="preserve">Framing inspection</t>
@@ -529,10 +541,10 @@
     <t xml:space="preserve">Framing Complete (30%)</t>
   </si>
   <si>
-    <t xml:space="preserve">Flat roofing, parapet flashing, skylight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prime Seal (roof) / skylight installer</t>
+    <t xml:space="preserve">Flat roofing, aluminum, downspouts, skylight curb + unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime Seal (roof + aluminum) / framer (skylight)</t>
   </si>
   <si>
     <t xml:space="preserve">Window install (client-supplied units)</t>
@@ -856,195 +868,270 @@
     <t xml:space="preserve">Fabiano's General Works line includes licensed electrical + ESA, batts, vapour barrier, drywall, MDF trim and paint. Hardwood, doors and hardware are client-supplied (install only).</t>
   </si>
   <si>
-    <t xml:space="preserve">439 Manning Ave: Leveling 2.0 (carried costs for the margin check)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As of Oct 22, 2026. Blue = carried amount set by Raff. Green = pulled from All Bids or Inputs. Windows and client finish materials are not in base cost.</t>
+    <t xml:space="preserve">439 Manning Ave: Leveling 2.0 (negotiated targets for the margin check)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As of Oct 25, 2026. Blue = typed-in number (Raff's negotiated target or an allowance). Green = pulled from All Bids or Inputs. Windows and client finish materials are not in base cost.</t>
   </si>
   <si>
     <t xml:space="preserve">Carried with</t>
   </si>
   <si>
-    <t xml:space="preserve">Basis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carried cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">At quoted price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variance vs budget</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gap to close (quoted - carried)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raff carry; Fabiano quoted $30,500</t>
+    <t xml:space="preserve">Scope / basis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quoted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required (negotiated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gap to negotiate (quoted - required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required vs budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negotiation note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General Works + Demolition (all-in)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GW $30,500 + demo $7,400 (bid #15). All-in must include the master closet drywall repair.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All-in target. Closet repair inside this number.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aryan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bid #31. Low bid now Comfort $13,000 (#68).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target $12,000. Ridge raise priced separately (row below).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONA (Jonathan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bid #43 lumber package</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carry $6,500. Walk-away max $7,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flat Roof + all aluminum + gutters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime Seal Roofing Systems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bid #53: roof, scuppers, collector boxes, downspouts, coping. Plus existing eavestrough/downspout tie-ins.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$6,000 with all aluminum + gutters. Elvis (Safety) re-pricing by Oct 26, 6 PM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bid #38: ~650 sq ft rear + ~300 sq ft north side, soffit/fascia, capping, WRB, flashing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target $7,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MiTech HVAC, Option 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quote #611: single zone 12k BTU $3,200 + vent runs $250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-confirm (quote expired). Client to be told it replaces the tie-in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FoamIt (Nadia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bid #13. Milan Insulation $2,372 (#54) also in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target $3,200.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stephenson's Rentals + United (toilet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scaffold $1,446 + hoist $3,731 + bins $2,800 (Stephenson's #66) + toilet $1,000 (United #64) + boom/deliveries $1,500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built up from the quoted monthly rates. JobTread shows $2,539 / $2,928, which are not the full rental.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ridge raise + re-shingle (if required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Framer + Prime Seal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contract: raise front ridge as required. Not priced by any trade yet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowance. Get it priced as a separate line; drop to $0 if La Vecchia confirms it is not needed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skylight unit + install (flat, den)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONA unit + framer install</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONA $289 (#61) + $250 install allowance. Opening framed, curb waterproofed by roofer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm the flat skylight is in the contract price (added May 24).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Winter protection / temporary heat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PalmView</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowance: tarps, poly, temporary heat while the roof is open in Jan to Feb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowance. Remove if demo moves to spring.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At quoted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At required (negotiated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target markup on cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope check (Oct 25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aluminum: new roof drainage, coping and existing eavestrough tie-ins carried by the roofer; soffit, fascia and window capping in Baz's siding scope.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Window count: Aryan's scope says 6 window openings; drawings, Baz and the other framers say 4. Confirm before framing award and window order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrical: HVAC Option 2 needs a 15A double-pole breaker, not the 30A in Fabiano's scope. Update his work order (small credit).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Side-wall cladding: designer to confirm vinyl is allowed at the side wall (limiting distance) before Baz orders.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Building permit fee: confirm whether the client pays the City directly (they paid the zoning fee).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not in base cost: windows (supply + install) and client finish materials (hardwood, interior doors, hardware). Add-ons priced separately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">439 Manning Ave: Bid Leveling Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yellow cells are the levers. Change them and every tab updates. Blue = typed-in number, black = formula, green = pulled from another tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source / note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contract sell: 2.0 Rear Addition (pre-HST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender Package, Margin Check (from invoice #22288). Excludes design fees and add-ons.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target markup on cost (SOP Step 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tendering SOP: cost target = contract sell / 1.35.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabiano General Works price (negotiated target)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raff's negotiation target, Oct 22. Fabiano quoted $30,500 for General Works (JobTread bid #15). Change to the agreed number.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does Fabiano's price include demolition? (Yes/No)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabiano priced demo as a separate line ($7,400), per the work order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demolition cost if separate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabiano demo line, JobTread bid #15 (Oct 22). Doctor Demo still pending.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roof + siding option (Split / Safety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split = lowest flat roof bid + lowest siding bid (now Prime Seal $5,900 + Baz $7,900). Safety = Safety Roofing combo $20,580 (siding, flat roof and skylight).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construction contingency (% of cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender Package: 10% budget reserve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender Package P2 provisional / change order risk.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Manning Bid Requests (from JobTread, Oct 25, 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amounts are the cost entered on each JobTread bid request. HST treatment not confirmed. To add a bid, insert a row above the last one and copy column E down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lookup key (formula)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JobTread #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General Works + Demo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renomar Inc (Olimpiu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General Works (excl. demo)</t>
   </si>
   <si>
     <t xml:space="preserve">Demolition</t>
   </si>
   <si>
-    <t xml:space="preserve">Fabiano bid as quoted (#15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TBD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raff estimate; low bid Aryan $14,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RONA (Jonathan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bid #43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prime Seal Roofing Systems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bid #53</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bid #38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MiTech HVAC, Option 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quote #611: single zone 12k BTU $3,200 + vent runs $250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FoamIt (Nadia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bid #13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PalmView direct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No quote yet: budget carried</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carried (2.0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">At quoted prices</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target markup on cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carried cost is the number we plan to buy each division at. 'At quoted price' uses the actual bids (Fabiano $30,500, framing low bid $14,000).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HVAC switches from tying into the existing mini-split (Option 1, $6,750) to a standalone 12,000 BTU single zone (Option 2, $3,450). Confirm with the client and MiTech.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Windows (supply + install) and client finish materials (hardwood, interior doors, hardware) are excluded from base cost.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site Services has no quote yet; the $11,500 budget is carried.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">439 Manning Ave: Bid Leveling Inputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellow cells are the levers. Change them and every tab updates. Blue = typed-in number, black = formula, green = pulled from another tab.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Input</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source / note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contract sell: 2.0 Rear Addition (pre-HST)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tender Package, Margin Check (from invoice #22288). Excludes design fees and add-ons.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target markup on cost (SOP Step 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tendering SOP: cost target = contract sell / 1.35.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabiano General Works price (negotiated target)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raff's negotiation target, Oct 22. Fabiano quoted $30,500 for General Works (JobTread bid #15). Change to the agreed number.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Does Fabiano's price include demolition? (Yes/No)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabiano priced demo as a separate line ($7,400), per the work order.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demolition cost if separate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabiano demo line, JobTread bid #15 (Oct 22). Doctor Demo still pending.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roof + siding option (Split / Safety)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Split</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Split = lowest flat roof bid + lowest siding bid (now Prime Seal $5,900 + Baz $7,900). Safety = Safety Roofing combo $20,580 (siding, flat roof and skylight).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Construction contingency (% of cost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tender Package: 10% budget reserve.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tender Package P2 provisional / change order risk.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All Manning Bid Requests (from JobTread, Oct 22, 2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amounts are the cost entered on each JobTread bid request. HST treatment not confirmed. To add a bid, insert a row above the last one and copy column E down.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vendor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amount ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lookup key (formula)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JobTread #</t>
-  </si>
-  <si>
-    <t xml:space="preserve">General Works + Demo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renomar Inc (Olimpiu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approved</t>
-  </si>
-  <si>
-    <t xml:space="preserve">General Works (excl. demo)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Doctor Demo (Roman)</t>
   </si>
   <si>
@@ -1063,9 +1150,6 @@
     <t xml:space="preserve">Framing</t>
   </si>
   <si>
-    <t xml:space="preserve">Aryan</t>
-  </si>
-  <si>
     <t xml:space="preserve">New Age Construction (Mario)</t>
   </si>
   <si>
@@ -1075,6 +1159,18 @@
     <t xml:space="preserve">JB Contracting (Jim)</t>
   </si>
   <si>
+    <t xml:space="preserve">Comfort Windows And Doors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novahaus Development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NA Contracting (Nelio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Golden Peak Construction (Edwin)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lumber</t>
   </si>
   <si>
@@ -1129,6 +1225,21 @@
     <t xml:space="preserve">Milan Insulation (Andy Cruz)</t>
   </si>
   <si>
+    <t xml:space="preserve">Site Services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stephenson's Rentals (Jehan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">United Rentals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skylight unit (flat, den)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONA (Rob Pianta)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Windows (client-paid)</t>
   </si>
   <si>
@@ -1145,6 +1256,15 @@
   </si>
   <si>
     <t xml:space="preserve">Amoroso Construction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masonry Professionals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red Robin Masonry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wallcent (Bryan)</t>
   </si>
   <si>
     <t xml:space="preserve">Add-on: Interior Brick</t>
@@ -1546,11 +1666,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2127,8 +2247,8 @@
         <v>40</v>
       </c>
       <c r="B26" s="8" t="n">
-        <f aca="false">'Leveling 2.0'!$E$20</f>
-        <v>82896.69</v>
+        <f aca="false">'Leveling 2.0'!$F$22</f>
+        <v>86516</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -2139,8 +2259,8 @@
         <v>41</v>
       </c>
       <c r="B27" s="8" t="n">
-        <f aca="false">'Leveling 2.0'!$F$20</f>
-        <v>90396.69</v>
+        <f aca="false">'Leveling 2.0'!$E$22</f>
+        <v>95012.69</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -2151,8 +2271,8 @@
         <v>42</v>
       </c>
       <c r="B28" s="9" t="n">
-        <f aca="false">'Leveling 2.0'!$E$23</f>
-        <v>0.273282282808802</v>
+        <f aca="false">'Leveling 2.0'!$F$25</f>
+        <v>0.241553432103095</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -2163,8 +2283,8 @@
         <v>43</v>
       </c>
       <c r="B29" s="9" t="n">
-        <f aca="false">'Leveling 2.0'!$F$23</f>
-        <v>0.207533181379854</v>
+        <f aca="false">'Leveling 2.0'!$E$25</f>
+        <v>0.167066801087052</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -2175,8 +2295,8 @@
         <v>44</v>
       </c>
       <c r="B30" s="9" t="n">
-        <f aca="false">'Leveling 2.0'!$E$32</f>
-        <v>0.156777776803717</v>
+        <f aca="false">'Leveling 2.0'!$F$34</f>
+        <v>0.121876041027439</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -3524,15 +3644,15 @@
         <v>30041</v>
       </c>
       <c r="C5" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"General Works (excl. demo)",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"General Works (excl. demo)",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>30500</v>
       </c>
       <c r="D5" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("General Works (excl. demo)|"&amp;ROUND(C5,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("General Works (excl. demo)|"&amp;ROUND(C5,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
         <v>FV Renovations (Fabiano)</v>
       </c>
       <c r="E5" s="26" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"General Works + Demo",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"General Works + Demo",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>57100</v>
       </c>
       <c r="F5" s="26" t="n">
@@ -3544,7 +3664,7 @@
         <v>-5041</v>
       </c>
       <c r="H5" s="35" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"General Works (excl. demo)",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$52,"General Works (excl. demo)",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="I5" s="27" t="n">
@@ -3559,11 +3679,11 @@
         <v>6290</v>
       </c>
       <c r="C6" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Demolition",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Demolition",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>7400</v>
       </c>
       <c r="D6" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Demolition|"&amp;ROUND(C6,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Demolition|"&amp;ROUND(C6,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
         <v>FV Renovations (Fabiano)</v>
       </c>
       <c r="E6" s="26" t="n">
@@ -3578,7 +3698,7 @@
         <v>1110</v>
       </c>
       <c r="H6" s="35" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Demolition",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$52,"Demolition",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="I6" s="27" t="n">
@@ -3593,28 +3713,28 @@
         <v>23128</v>
       </c>
       <c r="C7" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Framing",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
-        <v>14000</v>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Framing",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
+        <v>13000</v>
       </c>
       <c r="D7" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Framing|"&amp;ROUND(C7,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
-        <v>Aryan</v>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Framing|"&amp;ROUND(C7,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
+        <v>Comfort Windows And Doors</v>
       </c>
       <c r="E7" s="26" t="n">
         <f aca="false">C7</f>
-        <v>14000</v>
+        <v>13000</v>
       </c>
       <c r="F7" s="26" t="n">
         <f aca="false">E7</f>
-        <v>14000</v>
+        <v>13000</v>
       </c>
       <c r="G7" s="26" t="n">
         <f aca="false">F7-B7</f>
-        <v>-9128</v>
+        <v>-10128</v>
       </c>
       <c r="H7" s="35" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Framing",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$52,"Framing",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
+        <v>5</v>
       </c>
       <c r="I7" s="27" t="n">
         <v>3</v>
@@ -3628,11 +3748,11 @@
         <v>4900</v>
       </c>
       <c r="C8" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Lumber",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Lumber",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>6386.19</v>
       </c>
       <c r="D8" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Lumber|"&amp;ROUND(C8,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Lumber|"&amp;ROUND(C8,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
         <v>RONA (Jonathan)</v>
       </c>
       <c r="E8" s="26" t="n">
@@ -3648,7 +3768,7 @@
         <v>1486.19</v>
       </c>
       <c r="H8" s="35" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Lumber",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$52,"Lumber",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>3</v>
       </c>
       <c r="I8" s="27" t="n">
@@ -3663,11 +3783,11 @@
         <v>8010</v>
       </c>
       <c r="C9" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Flat Roofing",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Flat Roofing",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>5900</v>
       </c>
       <c r="D9" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Flat Roofing|"&amp;ROUND(C9,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Flat Roofing|"&amp;ROUND(C9,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
         <v>Prime Seal Roofing Systems (Ellery)</v>
       </c>
       <c r="E9" s="26" t="n">
@@ -3683,7 +3803,7 @@
         <v>-2110</v>
       </c>
       <c r="H9" s="35" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Flat Roofing",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$52,"Flat Roofing",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>2</v>
       </c>
       <c r="I9" s="27" t="n">
@@ -3698,11 +3818,11 @@
         <v>17750</v>
       </c>
       <c r="C10" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Siding",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Siding",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>7900</v>
       </c>
       <c r="D10" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Siding|"&amp;ROUND(C10,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Siding|"&amp;ROUND(C10,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
         <v>Baz Aluminum</v>
       </c>
       <c r="E10" s="26" t="n">
@@ -3718,7 +3838,7 @@
         <v>-9850</v>
       </c>
       <c r="H10" s="35" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Siding",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$52,"Siding",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="I10" s="27" t="n">
@@ -3733,11 +3853,11 @@
         <v>0</v>
       </c>
       <c r="C11" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Roof + Siding + Skylight Combo",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Roof + Siding + Skylight Combo",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>20580</v>
       </c>
       <c r="D11" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Roof + Siding + Skylight Combo|"&amp;ROUND(C11,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Roof + Siding + Skylight Combo|"&amp;ROUND(C11,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
         <v>Safety Roofing (Elvis)</v>
       </c>
       <c r="E11" s="26" t="n">
@@ -3753,7 +3873,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="35" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Roof + Siding + Skylight Combo",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$52,"Roof + Siding + Skylight Combo",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>1</v>
       </c>
       <c r="I11" s="27" t="n">
@@ -3768,11 +3888,11 @@
         <v>6750</v>
       </c>
       <c r="C12" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"HVAC",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"HVAC",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>9370</v>
       </c>
       <c r="D12" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("HVAC|"&amp;ROUND(C12,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("HVAC|"&amp;ROUND(C12,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
         <v>Ideal Heating (Leena)</v>
       </c>
       <c r="E12" s="26" t="n">
@@ -3788,7 +3908,7 @@
         <v>2620</v>
       </c>
       <c r="H12" s="35" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"HVAC",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$52,"HVAC",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>2</v>
       </c>
       <c r="I12" s="27" t="n">
@@ -3803,28 +3923,28 @@
         <v>3430</v>
       </c>
       <c r="C13" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Spray Foam",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
-        <v>3360.5</v>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Spray Foam",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
+        <v>2371.8</v>
       </c>
       <c r="D13" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Spray Foam|"&amp;ROUND(C13,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
-        <v>FoamIt (Nadia)</v>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Spray Foam|"&amp;ROUND(C13,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
+        <v>Milan Insulation (Andy Cruz)</v>
       </c>
       <c r="E13" s="26" t="n">
         <f aca="false">C13</f>
-        <v>3360.5</v>
+        <v>2371.8</v>
       </c>
       <c r="F13" s="26" t="n">
         <f aca="false">E13</f>
-        <v>3360.5</v>
+        <v>2371.8</v>
       </c>
       <c r="G13" s="26" t="n">
         <f aca="false">F13-B13</f>
-        <v>-69.5</v>
+        <v>-1058.2</v>
       </c>
       <c r="H13" s="35" t="n">
-        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$39,"Spray Foam",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS('All Bids'!$A$5:$A$52,"Spray Foam",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
+        <v>2</v>
       </c>
       <c r="I13" s="27" t="n">
         <v>3</v>
@@ -3874,15 +3994,15 @@
       <c r="D15" s="29"/>
       <c r="E15" s="31" t="n">
         <f aca="false">SUM(E5:E14)</f>
-        <v>115516.69</v>
+        <v>113527.99</v>
       </c>
       <c r="F15" s="31" t="n">
         <f aca="false">SUM(F5:F14)</f>
-        <v>90816.69</v>
+        <v>88827.99</v>
       </c>
       <c r="G15" s="31" t="n">
         <f aca="false">SUM(G5:G14)</f>
-        <v>-20982.31</v>
+        <v>-22971.01</v>
       </c>
       <c r="H15" s="29"/>
       <c r="I15" s="29"/>
@@ -3962,11 +4082,11 @@
       <c r="D20" s="2"/>
       <c r="E20" s="36" t="n">
         <f aca="false">E15</f>
-        <v>115516.69</v>
+        <v>113527.99</v>
       </c>
       <c r="F20" s="36" t="n">
         <f aca="false">F15</f>
-        <v>90816.69</v>
+        <v>88827.99</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -3981,11 +4101,11 @@
       <c r="D21" s="2"/>
       <c r="E21" s="37" t="n">
         <f aca="false">E20-E19</f>
-        <v>31020.3937037037</v>
+        <v>29031.6937037037</v>
       </c>
       <c r="F21" s="37" t="n">
         <f aca="false">F20-F19</f>
-        <v>6320.39370370371</v>
+        <v>4331.69370370371</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -4000,11 +4120,11 @@
       <c r="D22" s="2"/>
       <c r="E22" s="36" t="n">
         <f aca="false">E18-E20</f>
-        <v>-1446.69</v>
+        <v>542.009999999995</v>
       </c>
       <c r="F22" s="36" t="n">
         <f aca="false">F18-F20</f>
-        <v>23253.31</v>
+        <v>25242.01</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -4019,11 +4139,11 @@
       <c r="D23" s="2"/>
       <c r="E23" s="38" t="n">
         <f aca="false">IF(E18=0,0,E22/E18)</f>
-        <v>-0.0126824756728325</v>
+        <v>0.00475155606206711</v>
       </c>
       <c r="F23" s="38" t="n">
         <f aca="false">IF(F18=0,0,F22/F18)</f>
-        <v>0.203851231699833</v>
+        <v>0.221285263434733</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
@@ -4038,11 +4158,11 @@
       <c r="D24" s="2"/>
       <c r="E24" s="38" t="n">
         <f aca="false">IF(E20=0,0,E22/E20)</f>
-        <v>-0.012523644851666</v>
+        <v>0.00477424113648092</v>
       </c>
       <c r="F24" s="38" t="n">
         <f aca="false">IF(F20=0,0,F22/F20)</f>
-        <v>0.256046658384048</v>
+        <v>0.284167299068683</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -4100,11 +4220,11 @@
       <c r="D28" s="2"/>
       <c r="E28" s="36" t="n">
         <f aca="false">E20*Inputs!$B$11</f>
-        <v>11551.669</v>
+        <v>11352.799</v>
       </c>
       <c r="F28" s="36" t="n">
         <f aca="false">F20*Inputs!$B$11</f>
-        <v>9081.669</v>
+        <v>8882.799</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -4138,11 +4258,11 @@
       <c r="D30" s="2"/>
       <c r="E30" s="37" t="n">
         <f aca="false">E20+E28+E29</f>
-        <v>132068.359</v>
+        <v>129880.789</v>
       </c>
       <c r="F30" s="37" t="n">
         <f aca="false">F20+F28+F29</f>
-        <v>104898.359</v>
+        <v>102710.789</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -4157,11 +4277,11 @@
       <c r="D31" s="2"/>
       <c r="E31" s="36" t="n">
         <f aca="false">E18-E30</f>
-        <v>-17998.359</v>
+        <v>-15810.789</v>
       </c>
       <c r="F31" s="36" t="n">
         <f aca="false">F18-F30</f>
-        <v>9171.641</v>
+        <v>11359.211</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -4176,11 +4296,11 @@
       <c r="D32" s="2"/>
       <c r="E32" s="38" t="n">
         <f aca="false">IF(E18=0,0,E31/E18)</f>
-        <v>-0.15778345752608</v>
+        <v>-0.138606022617691</v>
       </c>
       <c r="F32" s="38" t="n">
         <f aca="false">IF(F18=0,0,F31/F18)</f>
-        <v>0.0804036205838521</v>
+        <v>0.0995810554922416</v>
       </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
@@ -4243,23 +4363,23 @@
         <v>36400</v>
       </c>
       <c r="C36" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Add-on: Brick Veneer",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
-        <v>31200</v>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Add-on: Brick Veneer",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
+        <v>8320</v>
       </c>
       <c r="D36" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Add-on: Brick Veneer|"&amp;ROUND(C36,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
-        <v>Amoroso Construction</v>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Add-on: Brick Veneer|"&amp;ROUND(C36,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
+        <v>Masonry Professionals</v>
       </c>
       <c r="E36" s="33" t="n">
         <v>8000</v>
       </c>
       <c r="F36" s="26" t="n">
         <f aca="false">C36*(1+Inputs!$B$6)</f>
-        <v>42120</v>
+        <v>11232</v>
       </c>
       <c r="G36" s="26" t="n">
         <f aca="false">F36-E36</f>
-        <v>34120</v>
+        <v>3232</v>
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -4272,23 +4392,23 @@
         <v>3960</v>
       </c>
       <c r="C37" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Add-on: Interior Brick",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
-        <v>10800</v>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Add-on: Interior Brick",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
+        <v>5850</v>
       </c>
       <c r="D37" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Add-on: Interior Brick|"&amp;ROUND(C37,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
-        <v>Amoroso Construction</v>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Add-on: Interior Brick|"&amp;ROUND(C37,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
+        <v>Masonry Professionals</v>
       </c>
       <c r="E37" s="33" t="n">
         <v>3600</v>
       </c>
       <c r="F37" s="26" t="n">
         <f aca="false">C37*(1+Inputs!$B$6)</f>
-        <v>14580</v>
+        <v>7897.5</v>
       </c>
       <c r="G37" s="26" t="n">
         <f aca="false">F37-E37</f>
-        <v>10980</v>
+        <v>4297.5</v>
       </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
@@ -4301,11 +4421,11 @@
         <v>4600</v>
       </c>
       <c r="C38" s="8" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Add-on: Skylight",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Add-on: Skylight",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>3300</v>
       </c>
       <c r="D38" s="34" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Add-on: Skylight|"&amp;ROUND(C38,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Add-on: Skylight|"&amp;ROUND(C38,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
         <v>Skylight Services Ltd</v>
       </c>
       <c r="E38" s="33" t="n">
@@ -4341,11 +4461,11 @@
         <v>8470</v>
       </c>
       <c r="C40" s="40" t="n">
-        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$39,'All Bids'!$A$5:$A$39,"Windows (client-paid)",'All Bids'!$C$5:$C$39,"Approved",'All Bids'!$D$5:$D$39,"&gt;0")</f>
+        <f aca="false">_xlfn.MINIFS('All Bids'!$D$5:$D$52,'All Bids'!$A$5:$A$52,"Windows (client-paid)",'All Bids'!$C$5:$C$52,"Approved",'All Bids'!$D$5:$D$52,"&gt;0")</f>
         <v>7850</v>
       </c>
       <c r="D40" s="41" t="str">
-        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$39,MATCH("Windows (client-paid)|"&amp;ROUND(C40,2),'All Bids'!$E$5:$E$39,0)),"No price yet")</f>
+        <f aca="false">IFERROR(INDEX('All Bids'!$B$5:$B$52,MATCH("Windows (client-paid)|"&amp;ROUND(C40,2),'All Bids'!$E$5:$E$52,0)),"No price yet")</f>
         <v>JS Windows and Doors</v>
       </c>
       <c r="E40" s="2"/>
@@ -4529,15 +4649,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4551,6 +4673,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -4563,6 +4686,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
@@ -4573,8 +4697,9 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
         <v>150</v>
       </c>
@@ -4599,627 +4724,711 @@
       <c r="H4" s="32" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
-        <v>159</v>
+      <c r="I4" s="32" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="42" t="s">
+        <v>215</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>92</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D5" s="33" t="n">
-        <v>30041</v>
-      </c>
-      <c r="E5" s="43" t="n">
-        <v>27000</v>
-      </c>
-      <c r="F5" s="8" t="n">
-        <f aca="false">'All Bids'!$D$6</f>
-        <v>30500</v>
+        <v>36331</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <f aca="false">'All Bids'!$D$6+'All Bids'!$D$7</f>
+        <v>37900</v>
+      </c>
+      <c r="F5" s="43" t="n">
+        <v>32250</v>
       </c>
       <c r="G5" s="26" t="n">
-        <f aca="false">E5-D5</f>
-        <v>-3041</v>
+        <f aca="false">E5-F5</f>
+        <v>5650</v>
       </c>
       <c r="H5" s="26" t="n">
-        <f aca="false">F5-E5</f>
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
-        <v>215</v>
+        <f aca="false">F5-D5</f>
+        <v>-4081</v>
+      </c>
+      <c r="I5" s="42" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="42" t="s">
+        <v>161</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>92</v>
+        <v>218</v>
       </c>
       <c r="C6" s="42" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>6290</v>
+        <v>23128</v>
       </c>
       <c r="E6" s="8" t="n">
-        <f aca="false">'All Bids'!$D$7</f>
-        <v>7400</v>
-      </c>
-      <c r="F6" s="36" t="n">
-        <f aca="false">E6</f>
-        <v>7400</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <f aca="false">E6-D6</f>
-        <v>1110</v>
-      </c>
-      <c r="H6" s="26" t="n">
-        <f aca="false">F6-E6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>161</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="C7" s="42" t="s">
-        <v>218</v>
-      </c>
-      <c r="D7" s="33" t="n">
-        <v>23128</v>
-      </c>
-      <c r="E7" s="43" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F7" s="8" t="n">
         <f aca="false">'All Bids'!$D$11</f>
         <v>14000</v>
       </c>
+      <c r="F6" s="43" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G6" s="26" t="n">
+        <f aca="false">E6-F6</f>
+        <v>2000</v>
+      </c>
+      <c r="H6" s="26" t="n">
+        <f aca="false">F6-D6</f>
+        <v>-11128</v>
+      </c>
+      <c r="I6" s="42" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="42" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="C7" s="42" t="s">
+        <v>222</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>4900</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <f aca="false">'All Bids'!$D$19</f>
+        <v>6386.19</v>
+      </c>
+      <c r="F7" s="43" t="n">
+        <v>6500</v>
+      </c>
       <c r="G7" s="26" t="n">
-        <f aca="false">E7-D7</f>
-        <v>-13128</v>
+        <f aca="false">E7-F7</f>
+        <v>-113.81</v>
       </c>
       <c r="H7" s="26" t="n">
-        <f aca="false">F7-E7</f>
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>162</v>
+        <f aca="false">F7-D7</f>
+        <v>1600</v>
+      </c>
+      <c r="I7" s="42" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="42" t="s">
+        <v>224</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="C8" s="42" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>4900</v>
+        <v>8010</v>
       </c>
       <c r="E8" s="8" t="n">
-        <f aca="false">'All Bids'!$D$15</f>
-        <v>6386.19</v>
-      </c>
-      <c r="F8" s="36" t="n">
-        <f aca="false">E8</f>
-        <v>6386.19</v>
+        <f aca="false">'All Bids'!$D$25</f>
+        <v>5900</v>
+      </c>
+      <c r="F8" s="43" t="n">
+        <v>6000</v>
       </c>
       <c r="G8" s="26" t="n">
-        <f aca="false">E8-D8</f>
-        <v>1486.19</v>
+        <f aca="false">E8-F8</f>
+        <v>-100</v>
       </c>
       <c r="H8" s="26" t="n">
-        <f aca="false">F8-E8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>163</v>
+        <f aca="false">F8-D8</f>
+        <v>-2010</v>
+      </c>
+      <c r="I8" s="42" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="42" t="s">
+        <v>164</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>221</v>
+        <v>102</v>
       </c>
       <c r="C9" s="42" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>8010</v>
+        <v>17750</v>
       </c>
       <c r="E9" s="8" t="n">
-        <f aca="false">'All Bids'!$D$21</f>
-        <v>5900</v>
-      </c>
-      <c r="F9" s="36" t="n">
-        <f aca="false">E9</f>
-        <v>5900</v>
+        <f aca="false">'All Bids'!$D$27</f>
+        <v>7900</v>
+      </c>
+      <c r="F9" s="43" t="n">
+        <v>7000</v>
       </c>
       <c r="G9" s="26" t="n">
-        <f aca="false">E9-D9</f>
-        <v>-2110</v>
+        <f aca="false">E9-F9</f>
+        <v>900</v>
       </c>
       <c r="H9" s="26" t="n">
-        <f aca="false">F9-E9</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
-        <v>164</v>
+        <f aca="false">F9-D9</f>
+        <v>-10750</v>
+      </c>
+      <c r="I9" s="42" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="42" t="s">
+        <v>166</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>102</v>
+        <v>230</v>
       </c>
       <c r="C10" s="42" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>17750</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <f aca="false">'All Bids'!$D$23</f>
-        <v>7900</v>
+        <v>6750</v>
+      </c>
+      <c r="E10" s="33" t="n">
+        <v>3450</v>
       </c>
       <c r="F10" s="36" t="n">
         <f aca="false">E10</f>
-        <v>7900</v>
+        <v>3450</v>
       </c>
       <c r="G10" s="26" t="n">
-        <f aca="false">E10-D10</f>
-        <v>-9850</v>
+        <f aca="false">E10-F10</f>
+        <v>0</v>
       </c>
       <c r="H10" s="26" t="n">
-        <f aca="false">F10-E10</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
-        <v>166</v>
+        <f aca="false">F10-D10</f>
+        <v>-3300</v>
+      </c>
+      <c r="I10" s="42" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="42" t="s">
+        <v>167</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C11" s="42" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>6750</v>
-      </c>
-      <c r="E11" s="43" t="n">
-        <v>3450</v>
-      </c>
-      <c r="F11" s="36" t="n">
-        <f aca="false">E11</f>
-        <v>3450</v>
+        <v>3430</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <f aca="false">'All Bids'!$D$34</f>
+        <v>3360.5</v>
+      </c>
+      <c r="F11" s="43" t="n">
+        <v>3200</v>
       </c>
       <c r="G11" s="26" t="n">
-        <f aca="false">E11-D11</f>
-        <v>-3300</v>
+        <f aca="false">E11-F11</f>
+        <v>160.5</v>
       </c>
       <c r="H11" s="26" t="n">
-        <f aca="false">F11-E11</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>167</v>
+        <f aca="false">F11-D11</f>
+        <v>-230</v>
+      </c>
+      <c r="I11" s="42" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="42" t="s">
+        <v>168</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="C12" s="42" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>3430</v>
-      </c>
-      <c r="E12" s="8" t="n">
-        <f aca="false">'All Bids'!$D$30</f>
-        <v>3360.5</v>
+        <v>11500</v>
+      </c>
+      <c r="E12" s="33" t="n">
+        <v>10477</v>
       </c>
       <c r="F12" s="36" t="n">
         <f aca="false">E12</f>
-        <v>3360.5</v>
+        <v>10477</v>
       </c>
       <c r="G12" s="26" t="n">
-        <f aca="false">E12-D12</f>
-        <v>-69.5</v>
+        <f aca="false">E12-F12</f>
+        <v>0</v>
       </c>
       <c r="H12" s="26" t="n">
-        <f aca="false">F12-E12</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
-        <v>168</v>
+        <f aca="false">F12-D12</f>
+        <v>-1023</v>
+      </c>
+      <c r="I12" s="42" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="42" t="s">
+        <v>239</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="C13" s="42" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>11500</v>
-      </c>
-      <c r="E13" s="36" t="n">
-        <f aca="false">D13</f>
-        <v>11500</v>
+        <v>3600</v>
+      </c>
+      <c r="E13" s="33" t="n">
+        <v>3600</v>
       </c>
       <c r="F13" s="36" t="n">
         <f aca="false">E13</f>
-        <v>11500</v>
+        <v>3600</v>
       </c>
       <c r="G13" s="26" t="n">
-        <f aca="false">E13-D13</f>
+        <f aca="false">E13-F13</f>
         <v>0</v>
       </c>
       <c r="H13" s="26" t="n">
-        <f aca="false">F13-E13</f>
+        <f aca="false">F13-D13</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="s">
+      <c r="I13" s="42" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="42" t="s">
+        <v>243</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="C14" s="42" t="s">
+        <v>245</v>
+      </c>
+      <c r="D14" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <f aca="false">'All Bids'!$D$38+250</f>
+        <v>539</v>
+      </c>
+      <c r="F14" s="36" t="n">
+        <f aca="false">E14</f>
+        <v>539</v>
+      </c>
+      <c r="G14" s="26" t="n">
+        <f aca="false">E14-F14</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="26" t="n">
+        <f aca="false">F14-D14</f>
+        <v>539</v>
+      </c>
+      <c r="I14" s="42" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="42" t="s">
+        <v>247</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>248</v>
+      </c>
+      <c r="C15" s="42" t="s">
+        <v>249</v>
+      </c>
+      <c r="D15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="33" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F15" s="36" t="n">
+        <f aca="false">E15</f>
+        <v>1500</v>
+      </c>
+      <c r="G15" s="26" t="n">
+        <f aca="false">E15-F15</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="26" t="n">
+        <f aca="false">F15-D15</f>
+        <v>1500</v>
+      </c>
+      <c r="I15" s="42" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="29" t="s">
         <v>170</v>
       </c>
-      <c r="B14" s="29"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="31" t="n">
-        <f aca="false">SUM(D5:D13)</f>
-        <v>111799</v>
-      </c>
-      <c r="E14" s="31" t="n">
-        <f aca="false">SUM(E5:E13)</f>
-        <v>82896.69</v>
-      </c>
-      <c r="F14" s="31" t="n">
-        <f aca="false">SUM(F5:F13)</f>
-        <v>90396.69</v>
-      </c>
-      <c r="G14" s="31" t="n">
-        <f aca="false">SUM(G5:G13)</f>
-        <v>-28902.31</v>
-      </c>
-      <c r="H14" s="31" t="n">
-        <f aca="false">SUM(H5:H13)</f>
-        <v>7500</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="31" t="n">
+        <f aca="false">SUM(D5:D15)</f>
+        <v>115399</v>
+      </c>
+      <c r="E16" s="31" t="n">
+        <f aca="false">SUM(E5:E15)</f>
+        <v>95012.69</v>
+      </c>
+      <c r="F16" s="31" t="n">
+        <f aca="false">SUM(F5:F15)</f>
+        <v>86516</v>
+      </c>
+      <c r="G16" s="31" t="n">
+        <f aca="false">SUM(G5:G15)</f>
+        <v>8496.69</v>
+      </c>
+      <c r="H16" s="31" t="n">
+        <f aca="false">SUM(H5:H15)</f>
+        <v>-28883</v>
+      </c>
+      <c r="I16" s="29"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="44" t="s">
-        <v>172</v>
-      </c>
+      <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="8" t="n">
-        <f aca="false">Inputs!$B$5</f>
-        <v>114070</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <f aca="false">Inputs!$B$5</f>
-        <v>114070</v>
-      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="9" t="n">
-        <f aca="false">Inputs!$B$6</f>
-        <v>0.35</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <f aca="false">Inputs!$B$6</f>
-        <v>0.35</v>
+      <c r="I17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>252</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="44" t="s">
-        <v>173</v>
+      <c r="A19" s="2" t="s">
+        <v>172</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
-      <c r="E19" s="36" t="n">
-        <f aca="false">E17/(1+E18)</f>
-        <v>84496.2962962963</v>
-      </c>
-      <c r="F19" s="36" t="n">
-        <f aca="false">F17/(1+F18)</f>
-        <v>84496.2962962963</v>
+      <c r="E19" s="8" t="n">
+        <f aca="false">Inputs!$B$5</f>
+        <v>114070</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <f aca="false">Inputs!$B$5</f>
+        <v>114070</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="44" t="s">
-        <v>174</v>
+      <c r="A20" s="2" t="s">
+        <v>253</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
-      <c r="E20" s="36" t="n">
-        <f aca="false">E14</f>
-        <v>82896.69</v>
-      </c>
-      <c r="F20" s="36" t="n">
-        <f aca="false">F14</f>
-        <v>90396.69</v>
+      <c r="E20" s="9" t="n">
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.35</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.35</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>175</v>
+      <c r="A21" s="2" t="s">
+        <v>173</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
-      <c r="E21" s="37" t="n">
-        <f aca="false">E20-E19</f>
-        <v>-1599.60629629629</v>
-      </c>
-      <c r="F21" s="37" t="n">
-        <f aca="false">F20-F19</f>
-        <v>5900.39370370371</v>
+      <c r="E21" s="36" t="n">
+        <f aca="false">E19/(1+E20)</f>
+        <v>84496.2962962963</v>
+      </c>
+      <c r="F21" s="36" t="n">
+        <f aca="false">F19/(1+F20)</f>
+        <v>84496.2962962963</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>176</v>
+      <c r="A22" s="2" t="s">
+        <v>174</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
-      <c r="E22" s="37" t="n">
-        <f aca="false">E17-E20</f>
-        <v>31173.31</v>
-      </c>
-      <c r="F22" s="37" t="n">
-        <f aca="false">F17-F20</f>
-        <v>23673.31</v>
+      <c r="E22" s="36" t="n">
+        <f aca="false">E16</f>
+        <v>95012.69</v>
+      </c>
+      <c r="F22" s="36" t="n">
+        <f aca="false">F16</f>
+        <v>86516</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
-      <c r="E23" s="38" t="n">
-        <f aca="false">IF(E17=0,0,E22/E17)</f>
-        <v>0.273282282808802</v>
-      </c>
-      <c r="F23" s="38" t="n">
-        <f aca="false">IF(F17=0,0,F22/F17)</f>
-        <v>0.207533181379854</v>
+      <c r="E23" s="37" t="n">
+        <f aca="false">E22-E21</f>
+        <v>10516.3937037037</v>
+      </c>
+      <c r="F23" s="37" t="n">
+        <f aca="false">F22-F21</f>
+        <v>2019.70370370371</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
-      <c r="E24" s="38" t="n">
-        <f aca="false">IF(E20=0,0,E22/E20)</f>
-        <v>0.376050117320728</v>
-      </c>
-      <c r="F24" s="38" t="n">
-        <f aca="false">IF(F20=0,0,F22/F20)</f>
-        <v>0.26188248706894</v>
+      <c r="E24" s="37" t="n">
+        <f aca="false">E19-E22</f>
+        <v>19057.31</v>
+      </c>
+      <c r="F24" s="37" t="n">
+        <f aca="false">F19-F22</f>
+        <v>27554</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="44" t="s">
-        <v>179</v>
+      <c r="A25" s="6" t="s">
+        <v>177</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
-      <c r="E25" s="45" t="n">
-        <f aca="false">E18/(1+E18)</f>
-        <v>0.259259259259259</v>
-      </c>
-      <c r="F25" s="45" t="n">
-        <f aca="false">F18/(1+F18)</f>
-        <v>0.259259259259259</v>
+      <c r="E25" s="38" t="n">
+        <f aca="false">IF(E19=0,0,E24/E19)</f>
+        <v>0.167066801087052</v>
+      </c>
+      <c r="F25" s="38" t="n">
+        <f aca="false">IF(F19=0,0,F24/F19)</f>
+        <v>0.241553432103095</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
+      <c r="A26" s="6" t="s">
+        <v>178</v>
+      </c>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
+      <c r="E26" s="38" t="n">
+        <f aca="false">IF(E22=0,0,E24/E22)</f>
+        <v>0.200576470364117</v>
+      </c>
+      <c r="F26" s="38" t="n">
+        <f aca="false">IF(F22=0,0,F24/F22)</f>
+        <v>0.318484442184105</v>
+      </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
-        <v>180</v>
+      <c r="A27" s="2" t="s">
+        <v>179</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
+      <c r="E27" s="44" t="n">
+        <f aca="false">E20/(1+E20)</f>
+        <v>0.259259259259259</v>
+      </c>
+      <c r="F27" s="44" t="n">
+        <f aca="false">F20/(1+F20)</f>
+        <v>0.259259259259259</v>
+      </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>181</v>
-      </c>
+      <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
-      <c r="E28" s="36" t="n">
-        <f aca="false">E20*Inputs!$B$11</f>
-        <v>8289.669</v>
-      </c>
-      <c r="F28" s="36" t="n">
-        <f aca="false">F20*Inputs!$B$11</f>
-        <v>9039.669</v>
-      </c>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>182</v>
+      <c r="A29" s="6" t="s">
+        <v>180</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
-      <c r="E29" s="8" t="n">
-        <f aca="false">Inputs!$B$12</f>
-        <v>5000</v>
-      </c>
-      <c r="F29" s="8" t="n">
-        <f aca="false">Inputs!$B$12</f>
-        <v>5000</v>
-      </c>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>183</v>
+      <c r="A30" s="2" t="s">
+        <v>181</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="37" t="n">
-        <f aca="false">E20+E28+E29</f>
-        <v>96186.359</v>
-      </c>
-      <c r="F30" s="37" t="n">
-        <f aca="false">F20+F28+F29</f>
-        <v>104436.359</v>
+      <c r="E30" s="36" t="n">
+        <f aca="false">E22*Inputs!$B$11</f>
+        <v>9501.269</v>
+      </c>
+      <c r="F30" s="36" t="n">
+        <f aca="false">F22*Inputs!$B$11</f>
+        <v>8651.6</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
-      <c r="E31" s="36" t="n">
-        <f aca="false">E17-E30</f>
-        <v>17883.641</v>
-      </c>
-      <c r="F31" s="36" t="n">
-        <f aca="false">F17-F30</f>
-        <v>9633.641</v>
+      <c r="E31" s="8" t="n">
+        <f aca="false">Inputs!$B$12</f>
+        <v>5000</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <f aca="false">Inputs!$B$12</f>
+        <v>5000</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="38" t="n">
-        <f aca="false">IF(E17=0,0,E31/E17)</f>
-        <v>0.156777776803717</v>
-      </c>
-      <c r="F32" s="38" t="n">
-        <f aca="false">IF(F17=0,0,F31/F17)</f>
-        <v>0.0844537652318752</v>
+      <c r="E32" s="37" t="n">
+        <f aca="false">E22+E30+E31</f>
+        <v>109513.959</v>
+      </c>
+      <c r="F32" s="37" t="n">
+        <f aca="false">F22+F30+F31</f>
+        <v>100167.6</v>
       </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2"/>
+      <c r="A33" s="2" t="s">
+        <v>184</v>
+      </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
+      <c r="E33" s="36" t="n">
+        <f aca="false">E19-E32</f>
+        <v>4556.041</v>
+      </c>
+      <c r="F33" s="36" t="n">
+        <f aca="false">F19-F32</f>
+        <v>13902.4</v>
+      </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
+      <c r="E34" s="38" t="n">
+        <f aca="false">IF(E19=0,0,E33/E19)</f>
+        <v>0.0399407469097922</v>
+      </c>
+      <c r="F34" s="38" t="n">
+        <f aca="false">IF(F19=0,0,F33/F19)</f>
+        <v>0.121876041027439</v>
+      </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12" t="s">
-        <v>233</v>
-      </c>
+      <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -5227,10 +5436,11 @@
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12" t="s">
-        <v>234</v>
+      <c r="A36" s="6" t="s">
+        <v>254</v>
       </c>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -5239,10 +5449,11 @@
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>235</v>
+        <v>255</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -5251,10 +5462,11 @@
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -5263,9 +5475,62 @@
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G5:G14">
+  <conditionalFormatting sqref="H5:H16">
     <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -5273,11 +5538,16 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E21:F21">
-    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+  <conditionalFormatting sqref="G5:G16">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="lessThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23:F23">
+    <cfRule type="cellIs" priority="5" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="lessThanOrEqual" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5307,14 +5577,14 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>237</v>
+        <v>261</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>238</v>
+        <v>262</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5326,101 +5596,101 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>239</v>
+        <v>263</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>240</v>
+        <v>264</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>241</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="44" t="s">
-        <v>242</v>
+      <c r="A5" s="45" t="s">
+        <v>266</v>
       </c>
       <c r="B5" s="43" t="n">
         <v>114070</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>243</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="44" t="s">
-        <v>244</v>
+      <c r="A6" s="45" t="s">
+        <v>268</v>
       </c>
       <c r="B6" s="46" t="n">
         <v>0.35</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>245</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="44" t="s">
-        <v>246</v>
+      <c r="A7" s="45" t="s">
+        <v>270</v>
       </c>
       <c r="B7" s="43" t="n">
         <v>25000</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>247</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="44" t="s">
-        <v>248</v>
+      <c r="A8" s="45" t="s">
+        <v>272</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>249</v>
+        <v>273</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>250</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="44" t="s">
-        <v>251</v>
+      <c r="A9" s="45" t="s">
+        <v>275</v>
       </c>
       <c r="B9" s="43" t="n">
         <v>7400</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>252</v>
+        <v>276</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="44" t="s">
-        <v>253</v>
+      <c r="A10" s="45" t="s">
+        <v>277</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>255</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="44" t="s">
-        <v>256</v>
+      <c r="A11" s="45" t="s">
+        <v>280</v>
       </c>
       <c r="B11" s="46" t="n">
         <v>0.1</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>257</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="44" t="s">
+      <c r="A12" s="45" t="s">
         <v>182</v>
       </c>
       <c r="B12" s="43" t="n">
         <v>5000</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>258</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -5449,7 +5719,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="32"/>
@@ -5461,7 +5731,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>259</v>
+        <v>283</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5471,7 +5741,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5492,30 +5762,30 @@
         <v>150</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>261</v>
+        <v>285</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>20</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>262</v>
+        <v>286</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>263</v>
+        <v>287</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>265</v>
+        <v>289</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>266</v>
+        <v>290</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D5" s="33" t="n">
         <v>57100</v>
@@ -5530,13 +5800,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>268</v>
+        <v>292</v>
       </c>
       <c r="B6" s="21" t="s">
         <v>92</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D6" s="33" t="n">
         <v>30500</v>
@@ -5551,13 +5821,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>215</v>
+        <v>293</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>92</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D7" s="33" t="n">
         <v>7400</v>
@@ -5572,13 +5842,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>215</v>
+        <v>293</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>269</v>
+        <v>294</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>270</v>
+        <v>295</v>
       </c>
       <c r="D8" s="33" t="n">
         <v>0</v>
@@ -5593,13 +5863,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>215</v>
+        <v>293</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>271</v>
+        <v>296</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>272</v>
+        <v>297</v>
       </c>
       <c r="D9" s="33" t="n">
         <v>0</v>
@@ -5614,13 +5884,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>215</v>
+        <v>293</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>273</v>
+        <v>298</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>272</v>
+        <v>297</v>
       </c>
       <c r="D10" s="33" t="n">
         <v>0</v>
@@ -5635,13 +5905,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>274</v>
+        <v>299</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>275</v>
+        <v>218</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D11" s="33" t="n">
         <v>14000</v>
@@ -5656,13 +5926,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>274</v>
+        <v>299</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>276</v>
+        <v>300</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>270</v>
+        <v>295</v>
       </c>
       <c r="D12" s="33" t="n">
         <v>0</v>
@@ -5677,13 +5947,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>274</v>
+        <v>299</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>277</v>
+        <v>301</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>272</v>
+        <v>297</v>
       </c>
       <c r="D13" s="33" t="n">
         <v>0</v>
@@ -5698,13 +5968,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>274</v>
+        <v>299</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>278</v>
+        <v>302</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>270</v>
+        <v>295</v>
       </c>
       <c r="D14" s="33" t="n">
         <v>0</v>
@@ -5719,149 +5989,149 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>279</v>
+        <v>299</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>219</v>
+        <v>303</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D15" s="33" t="n">
-        <v>6386.19</v>
+        <v>13000</v>
       </c>
       <c r="E15" s="18" t="str">
         <f aca="false">IF(AND(C15="Approved",D15&gt;0),A15&amp;"|"&amp;ROUND(D15,2),"")</f>
-        <v>Lumber|6386.19</v>
+        <v>Framing|13000</v>
       </c>
       <c r="F15" s="27" t="n">
-        <v>43</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>279</v>
+        <v>299</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>280</v>
+        <v>304</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D16" s="33" t="n">
-        <v>7040</v>
+        <v>15000</v>
       </c>
       <c r="E16" s="18" t="str">
         <f aca="false">IF(AND(C16="Approved",D16&gt;0),A16&amp;"|"&amp;ROUND(D16,2),"")</f>
-        <v>Lumber|7040</v>
+        <v>Framing|15000</v>
       </c>
       <c r="F16" s="27" t="n">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>279</v>
+        <v>299</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>281</v>
+        <v>305</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D17" s="33" t="n">
-        <v>7208.9</v>
+        <v>27700</v>
       </c>
       <c r="E17" s="18" t="str">
         <f aca="false">IF(AND(C17="Approved",D17&gt;0),A17&amp;"|"&amp;ROUND(D17,2),"")</f>
-        <v>Lumber|7208.9</v>
+        <v>Framing|27700</v>
       </c>
       <c r="F17" s="27" t="n">
-        <v>45</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>163</v>
+        <v>299</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D18" s="33" t="n">
-        <v>15700</v>
+        <v>29500</v>
       </c>
       <c r="E18" s="18" t="str">
         <f aca="false">IF(AND(C18="Approved",D18&gt;0),A18&amp;"|"&amp;ROUND(D18,2),"")</f>
-        <v>Flat Roofing|15700</v>
+        <v>Framing|29500</v>
       </c>
       <c r="F18" s="27" t="n">
-        <v>21</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>163</v>
+        <v>307</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>283</v>
+        <v>221</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>272</v>
+        <v>291</v>
       </c>
       <c r="D19" s="33" t="n">
-        <v>0</v>
+        <v>6386.19</v>
       </c>
       <c r="E19" s="18" t="str">
         <f aca="false">IF(AND(C19="Approved",D19&gt;0),A19&amp;"|"&amp;ROUND(D19,2),"")</f>
-        <v/>
+        <v>Lumber|6386.19</v>
       </c>
       <c r="F19" s="27" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="21" t="s">
-        <v>163</v>
+        <v>307</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>284</v>
+        <v>308</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>272</v>
+        <v>291</v>
       </c>
       <c r="D20" s="33" t="n">
-        <v>0</v>
+        <v>7040</v>
       </c>
       <c r="E20" s="18" t="str">
         <f aca="false">IF(AND(C20="Approved",D20&gt;0),A20&amp;"|"&amp;ROUND(D20,2),"")</f>
-        <v/>
+        <v>Lumber|7040</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="21" t="s">
-        <v>163</v>
+        <v>307</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>285</v>
+        <v>309</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D21" s="33" t="n">
-        <v>5900</v>
+        <v>7208.9</v>
       </c>
       <c r="E21" s="18" t="str">
         <f aca="false">IF(AND(C21="Approved",D21&gt;0),A21&amp;"|"&amp;ROUND(D21,2),"")</f>
-        <v>Flat Roofing|5900</v>
+        <v>Lumber|7208.9</v>
       </c>
       <c r="F21" s="27" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5869,52 +6139,52 @@
         <v>163</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>286</v>
+        <v>310</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>270</v>
+        <v>291</v>
       </c>
       <c r="D22" s="33" t="n">
-        <v>0</v>
+        <v>15700</v>
       </c>
       <c r="E22" s="18" t="str">
         <f aca="false">IF(AND(C22="Approved",D22&gt;0),A22&amp;"|"&amp;ROUND(D22,2),"")</f>
-        <v/>
+        <v>Flat Roofing|15700</v>
       </c>
       <c r="F22" s="27" t="n">
-        <v>56</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>287</v>
+        <v>163</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>102</v>
+        <v>311</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>267</v>
+        <v>297</v>
       </c>
       <c r="D23" s="33" t="n">
-        <v>7900</v>
+        <v>0</v>
       </c>
       <c r="E23" s="18" t="str">
         <f aca="false">IF(AND(C23="Approved",D23&gt;0),A23&amp;"|"&amp;ROUND(D23,2),"")</f>
-        <v>Siding|7900</v>
+        <v/>
       </c>
       <c r="F23" s="27" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>287</v>
+        <v>163</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>288</v>
+        <v>312</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>272</v>
+        <v>297</v>
       </c>
       <c r="D24" s="33" t="n">
         <v>0</v>
@@ -5924,81 +6194,81 @@
         <v/>
       </c>
       <c r="F24" s="27" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>289</v>
+        <v>163</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>290</v>
+        <v>313</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D25" s="33" t="n">
-        <v>20580</v>
+        <v>5900</v>
       </c>
       <c r="E25" s="18" t="str">
         <f aca="false">IF(AND(C25="Approved",D25&gt;0),A25&amp;"|"&amp;ROUND(D25,2),"")</f>
-        <v>Roof + Siding + Skylight Combo|20580</v>
+        <v>Flat Roofing|5900</v>
       </c>
       <c r="F25" s="27" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>291</v>
+        <v>163</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>292</v>
+        <v>314</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>267</v>
+        <v>295</v>
       </c>
       <c r="D26" s="33" t="n">
-        <v>9370</v>
+        <v>0</v>
       </c>
       <c r="E26" s="18" t="str">
         <f aca="false">IF(AND(C26="Approved",D26&gt;0),A26&amp;"|"&amp;ROUND(D26,2),"")</f>
-        <v>HVAC|9370</v>
+        <v/>
       </c>
       <c r="F26" s="27" t="n">
-        <v>28</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
+        <v>315</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>291</v>
       </c>
-      <c r="B27" s="21" t="s">
-        <v>293</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>267</v>
-      </c>
       <c r="D27" s="33" t="n">
-        <v>9950</v>
+        <v>7900</v>
       </c>
       <c r="E27" s="18" t="str">
         <f aca="false">IF(AND(C27="Approved",D27&gt;0),A27&amp;"|"&amp;ROUND(D27,2),"")</f>
-        <v>HVAC|9950</v>
+        <v>Siding|7900</v>
       </c>
       <c r="F27" s="27" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>291</v>
+        <v>315</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>294</v>
+        <v>316</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>272</v>
+        <v>297</v>
       </c>
       <c r="D28" s="33" t="n">
         <v>0</v>
@@ -6008,237 +6278,510 @@
         <v/>
       </c>
       <c r="F28" s="27" t="n">
-        <v>27</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
+        <v>317</v>
+      </c>
+      <c r="B29" s="21" t="s">
+        <v>318</v>
+      </c>
+      <c r="C29" s="21" t="s">
         <v>291</v>
       </c>
-      <c r="B29" s="21" t="s">
-        <v>295</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>272</v>
-      </c>
       <c r="D29" s="33" t="n">
-        <v>0</v>
+        <v>20580</v>
       </c>
       <c r="E29" s="18" t="str">
         <f aca="false">IF(AND(C29="Approved",D29&gt;0),A29&amp;"|"&amp;ROUND(D29,2),"")</f>
-        <v/>
+        <v>Roof + Siding + Skylight Combo|20580</v>
       </c>
       <c r="F29" s="27" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
-        <v>167</v>
+        <v>319</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>226</v>
+        <v>320</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D30" s="33" t="n">
-        <v>3360.5</v>
+        <v>9370</v>
       </c>
       <c r="E30" s="18" t="str">
         <f aca="false">IF(AND(C30="Approved",D30&gt;0),A30&amp;"|"&amp;ROUND(D30,2),"")</f>
-        <v>Spray Foam|3360.5</v>
+        <v>HVAC|9370</v>
       </c>
       <c r="F30" s="27" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>167</v>
+        <v>319</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>296</v>
+        <v>321</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>270</v>
+        <v>291</v>
       </c>
       <c r="D31" s="33" t="n">
-        <v>0</v>
+        <v>9950</v>
       </c>
       <c r="E31" s="18" t="str">
         <f aca="false">IF(AND(C31="Approved",D31&gt;0),A31&amp;"|"&amp;ROUND(D31,2),"")</f>
-        <v/>
+        <v>HVAC|9950</v>
       </c>
       <c r="F31" s="27" t="n">
-        <v>54</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
+        <v>319</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>322</v>
+      </c>
+      <c r="C32" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="B32" s="21" t="s">
-        <v>298</v>
-      </c>
-      <c r="C32" s="21" t="s">
-        <v>267</v>
-      </c>
       <c r="D32" s="33" t="n">
-        <v>7850</v>
+        <v>0</v>
       </c>
       <c r="E32" s="18" t="str">
         <f aca="false">IF(AND(C32="Approved",D32&gt;0),A32&amp;"|"&amp;ROUND(D32,2),"")</f>
-        <v>Windows (client-paid)|7850</v>
+        <v/>
       </c>
       <c r="F32" s="27" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="21" t="s">
+        <v>319</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>323</v>
+      </c>
+      <c r="C33" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="B33" s="21" t="s">
-        <v>299</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>267</v>
-      </c>
       <c r="D33" s="33" t="n">
-        <v>8340</v>
+        <v>0</v>
       </c>
       <c r="E33" s="18" t="str">
         <f aca="false">IF(AND(C33="Approved",D33&gt;0),A33&amp;"|"&amp;ROUND(D33,2),"")</f>
-        <v>Windows (client-paid)|8340</v>
+        <v/>
       </c>
       <c r="F33" s="27" t="n">
-        <v>47</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="21" t="s">
-        <v>297</v>
+        <v>167</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>300</v>
+        <v>233</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D34" s="33" t="n">
-        <v>9646.02</v>
+        <v>3360.5</v>
       </c>
       <c r="E34" s="18" t="str">
         <f aca="false">IF(AND(C34="Approved",D34&gt;0),A34&amp;"|"&amp;ROUND(D34,2),"")</f>
-        <v>Windows (client-paid)|9646.02</v>
+        <v>Spray Foam|3360.5</v>
       </c>
       <c r="F34" s="27" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="21" t="s">
-        <v>301</v>
+        <v>167</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>302</v>
+        <v>324</v>
       </c>
       <c r="C35" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D35" s="33" t="n">
-        <v>31200</v>
+        <v>2371.8</v>
       </c>
       <c r="E35" s="18" t="str">
         <f aca="false">IF(AND(C35="Approved",D35&gt;0),A35&amp;"|"&amp;ROUND(D35,2),"")</f>
-        <v>Add-on: Brick Veneer|31200</v>
+        <v>Spray Foam|2371.8</v>
       </c>
       <c r="F35" s="27" t="n">
-        <v>12</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="21" t="s">
-        <v>303</v>
+        <v>325</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>302</v>
+        <v>326</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D36" s="33" t="n">
-        <v>10800</v>
+        <v>2539</v>
       </c>
       <c r="E36" s="18" t="str">
         <f aca="false">IF(AND(C36="Approved",D36&gt;0),A36&amp;"|"&amp;ROUND(D36,2),"")</f>
-        <v>Add-on: Interior Brick|10800</v>
+        <v>Site Services|2539</v>
       </c>
       <c r="F36" s="27" t="n">
-        <v>14</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="21" t="s">
-        <v>304</v>
+        <v>325</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>305</v>
+        <v>327</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D37" s="33" t="n">
-        <v>3300</v>
+        <v>2928</v>
       </c>
       <c r="E37" s="18" t="str">
         <f aca="false">IF(AND(C37="Approved",D37&gt;0),A37&amp;"|"&amp;ROUND(D37,2),"")</f>
-        <v>Add-on: Skylight|3300</v>
+        <v>Site Services|2928</v>
       </c>
       <c r="F37" s="27" t="n">
-        <v>24</v>
+        <v>64</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="21" t="s">
-        <v>304</v>
+        <v>328</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>306</v>
+        <v>329</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>307</v>
+        <v>291</v>
       </c>
       <c r="D38" s="33" t="n">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="E38" s="18" t="str">
         <f aca="false">IF(AND(C38="Approved",D38&gt;0),A38&amp;"|"&amp;ROUND(D38,2),"")</f>
-        <v/>
+        <v>Skylight unit (flat, den)|289</v>
       </c>
       <c r="F38" s="27" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="21" t="s">
-        <v>308</v>
+        <v>330</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>267</v>
+        <v>291</v>
       </c>
       <c r="D39" s="33" t="n">
-        <v>1215</v>
+        <v>7850</v>
       </c>
       <c r="E39" s="18" t="str">
         <f aca="false">IF(AND(C39="Approved",D39&gt;0),A39&amp;"|"&amp;ROUND(D39,2),"")</f>
+        <v>Windows (client-paid)|7850</v>
+      </c>
+      <c r="F39" s="27" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="21" t="s">
+        <v>330</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>332</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D40" s="33" t="n">
+        <v>8340</v>
+      </c>
+      <c r="E40" s="18" t="str">
+        <f aca="false">IF(AND(C40="Approved",D40&gt;0),A40&amp;"|"&amp;ROUND(D40,2),"")</f>
+        <v>Windows (client-paid)|8340</v>
+      </c>
+      <c r="F40" s="27" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="21" t="s">
+        <v>330</v>
+      </c>
+      <c r="B41" s="21" t="s">
+        <v>333</v>
+      </c>
+      <c r="C41" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D41" s="33" t="n">
+        <v>9646.02</v>
+      </c>
+      <c r="E41" s="18" t="str">
+        <f aca="false">IF(AND(C41="Approved",D41&gt;0),A41&amp;"|"&amp;ROUND(D41,2),"")</f>
+        <v>Windows (client-paid)|9646.02</v>
+      </c>
+      <c r="F41" s="27" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="21" t="s">
+        <v>334</v>
+      </c>
+      <c r="B42" s="21" t="s">
+        <v>335</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D42" s="33" t="n">
+        <v>31200</v>
+      </c>
+      <c r="E42" s="18" t="str">
+        <f aca="false">IF(AND(C42="Approved",D42&gt;0),A42&amp;"|"&amp;ROUND(D42,2),"")</f>
+        <v>Add-on: Brick Veneer|31200</v>
+      </c>
+      <c r="F42" s="27" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="21" t="s">
+        <v>334</v>
+      </c>
+      <c r="B43" s="21" t="s">
+        <v>336</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D43" s="33" t="n">
+        <v>8320</v>
+      </c>
+      <c r="E43" s="18" t="str">
+        <f aca="false">IF(AND(C43="Approved",D43&gt;0),A43&amp;"|"&amp;ROUND(D43,2),"")</f>
+        <v>Add-on: Brick Veneer|8320</v>
+      </c>
+      <c r="F43" s="27" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21" t="s">
+        <v>334</v>
+      </c>
+      <c r="B44" s="21" t="s">
+        <v>337</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D44" s="33" t="n">
+        <v>16000</v>
+      </c>
+      <c r="E44" s="18" t="str">
+        <f aca="false">IF(AND(C44="Approved",D44&gt;0),A44&amp;"|"&amp;ROUND(D44,2),"")</f>
+        <v>Add-on: Brick Veneer|16000</v>
+      </c>
+      <c r="F44" s="27" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21" t="s">
+        <v>334</v>
+      </c>
+      <c r="B45" s="21" t="s">
+        <v>338</v>
+      </c>
+      <c r="C45" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="D45" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="18" t="str">
+        <f aca="false">IF(AND(C45="Approved",D45&gt;0),A45&amp;"|"&amp;ROUND(D45,2),"")</f>
+        <v/>
+      </c>
+      <c r="F45" s="27" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21" t="s">
+        <v>339</v>
+      </c>
+      <c r="B46" s="21" t="s">
+        <v>335</v>
+      </c>
+      <c r="C46" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D46" s="33" t="n">
+        <v>10800</v>
+      </c>
+      <c r="E46" s="18" t="str">
+        <f aca="false">IF(AND(C46="Approved",D46&gt;0),A46&amp;"|"&amp;ROUND(D46,2),"")</f>
+        <v>Add-on: Interior Brick|10800</v>
+      </c>
+      <c r="F46" s="27" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="21" t="s">
+        <v>339</v>
+      </c>
+      <c r="B47" s="21" t="s">
+        <v>336</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D47" s="33" t="n">
+        <v>5850</v>
+      </c>
+      <c r="E47" s="18" t="str">
+        <f aca="false">IF(AND(C47="Approved",D47&gt;0),A47&amp;"|"&amp;ROUND(D47,2),"")</f>
+        <v>Add-on: Interior Brick|5850</v>
+      </c>
+      <c r="F47" s="27" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="21" t="s">
+        <v>339</v>
+      </c>
+      <c r="B48" s="21" t="s">
+        <v>337</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D48" s="33" t="n">
+        <v>11250</v>
+      </c>
+      <c r="E48" s="18" t="str">
+        <f aca="false">IF(AND(C48="Approved",D48&gt;0),A48&amp;"|"&amp;ROUND(D48,2),"")</f>
+        <v>Add-on: Interior Brick|11250</v>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="21" t="s">
+        <v>339</v>
+      </c>
+      <c r="B49" s="21" t="s">
+        <v>338</v>
+      </c>
+      <c r="C49" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="D49" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="18" t="str">
+        <f aca="false">IF(AND(C49="Approved",D49&gt;0),A49&amp;"|"&amp;ROUND(D49,2),"")</f>
+        <v/>
+      </c>
+      <c r="F49" s="27" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="21" t="s">
+        <v>340</v>
+      </c>
+      <c r="B50" s="21" t="s">
+        <v>341</v>
+      </c>
+      <c r="C50" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D50" s="33" t="n">
+        <v>3300</v>
+      </c>
+      <c r="E50" s="18" t="str">
+        <f aca="false">IF(AND(C50="Approved",D50&gt;0),A50&amp;"|"&amp;ROUND(D50,2),"")</f>
+        <v>Add-on: Skylight|3300</v>
+      </c>
+      <c r="F50" s="27" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="21" t="s">
+        <v>340</v>
+      </c>
+      <c r="B51" s="21" t="s">
+        <v>342</v>
+      </c>
+      <c r="C51" s="21" t="s">
+        <v>343</v>
+      </c>
+      <c r="D51" s="33" t="n">
+        <v>300</v>
+      </c>
+      <c r="E51" s="18" t="str">
+        <f aca="false">IF(AND(C51="Approved",D51&gt;0),A51&amp;"|"&amp;ROUND(D51,2),"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="27" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="21" t="s">
+        <v>344</v>
+      </c>
+      <c r="B52" s="21" t="s">
+        <v>345</v>
+      </c>
+      <c r="C52" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="D52" s="33" t="n">
+        <v>1215</v>
+      </c>
+      <c r="E52" s="18" t="str">
+        <f aca="false">IF(AND(C52="Approved",D52&gt;0),A52&amp;"|"&amp;ROUND(D52,2),"")</f>
         <v>Hardwood Install (in GW scope)|1215</v>
       </c>
-      <c r="F39" s="27" t="n">
+      <c r="F52" s="27" t="n">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Manning Leveling 2.0: carry Milan Insulation for spray foam
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY6xq9eh2BK6Au4SE2w7Bc
</commit_message>
<xml_diff>
--- a/Manning_Construction_Plan.xlsx
+++ b/Manning_Construction_Plan.xlsx
@@ -397,7 +397,7 @@
     <t xml:space="preserve">1.</t>
   </si>
   <si>
-    <t xml:space="preserve">Negotiation targets (Leveling 2.0): Fabiano all-in $32,250 (quoted $37,900), Aryan $12,000 ($14,000), Baz $7,000 ($7,900), spray foam $3,200, RONA $6,500 (max $7,000), Prime Seal $6,000 with aluminum.</t>
+    <t xml:space="preserve">Negotiation targets (Leveling 2.0): Fabiano all-in $32,250 (quoted $37,900), Aryan $12,000 ($14,000), Baz $7,000 ($7,900), RONA $6,500 (max $7,000), Prime Seal $6,000 with aluminum. Spray foam: Milan at $2,372.</t>
   </si>
   <si>
     <t xml:space="preserve">2.</t>
@@ -949,280 +949,280 @@
     <t xml:space="preserve">Re-confirm (quote expired). Client to be told it replaces the tie-in.</t>
   </si>
   <si>
+    <t xml:space="preserve">Milan Insulation (Andy Cruz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bid #54. FoamIt $3,361 (#13) also in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carry Milan at quoted. Confirm full scope incl. sealing the third floor during spraying (occupied home).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stephenson's Rentals + United (toilet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scaffold $1,446 + hoist $3,731 + bins $2,800 (Stephenson's #66) + toilet $1,000 (United #64) + boom/deliveries $1,500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built up from the quoted monthly rates. JobTread shows $2,539 / $2,928, which are not the full rental.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ridge raise + re-shingle (if required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Framer + Prime Seal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contract: raise front ridge as required. Not priced by any trade yet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowance. Get it priced as a separate line; drop to $0 if La Vecchia confirms it is not needed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skylight unit + install (flat, den)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONA unit + framer install</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RONA $289 (#61) + $250 install allowance. Opening framed, curb waterproofed by roofer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm the flat skylight is in the contract price (added May 24).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Winter protection / temporary heat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PalmView</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowance: tarps, poly, temporary heat while the roof is open in Jan to Feb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowance. Remove if demo moves to spring.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At quoted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At required (negotiated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target markup on cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope check (Oct 25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aluminum: new roof drainage, coping and existing eavestrough tie-ins carried by the roofer; soffit, fascia and window capping in Baz's siding scope.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Window count: Aryan's scope says 6 window openings; drawings, Baz and the other framers say 4. Confirm before framing award and window order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrical: HVAC Option 2 needs a 15A double-pole breaker, not the 30A in Fabiano's scope. Update his work order (small credit).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Side-wall cladding: designer to confirm vinyl is allowed at the side wall (limiting distance) before Baz orders.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Building permit fee: confirm whether the client pays the City directly (they paid the zoning fee).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not in base cost: windows (supply + install) and client finish materials (hardwood, interior doors, hardware). Add-ons priced separately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">439 Manning Ave: Bid Leveling Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yellow cells are the levers. Change them and every tab updates. Blue = typed-in number, black = formula, green = pulled from another tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source / note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contract sell: 2.0 Rear Addition (pre-HST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender Package, Margin Check (from invoice #22288). Excludes design fees and add-ons.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target markup on cost (SOP Step 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tendering SOP: cost target = contract sell / 1.35.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabiano General Works price (negotiated target)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raff's negotiation target, Oct 22. Fabiano quoted $30,500 for General Works (JobTread bid #15). Change to the agreed number.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does Fabiano's price include demolition? (Yes/No)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabiano priced demo as a separate line ($7,400), per the work order.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demolition cost if separate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabiano demo line, JobTread bid #15 (Oct 22). Doctor Demo still pending.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roof + siding option (Split / Safety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split = lowest flat roof bid + lowest siding bid (now Prime Seal $5,900 + Baz $7,900). Safety = Safety Roofing combo $20,580 (siding, flat roof and skylight).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construction contingency (% of cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender Package: 10% budget reserve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender Package P2 provisional / change order risk.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Manning Bid Requests (from JobTread, Oct 25, 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amounts are the cost entered on each JobTread bid request. HST treatment not confirmed. To add a bid, insert a row above the last one and copy column E down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lookup key (formula)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JobTread #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General Works + Demo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renomar Inc (Olimpiu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General Works (excl. demo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demolition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doctor Demo (Roman)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bradley Demolition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Declined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universal Impact Services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Framing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Age Construction (Mario)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bogdan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JB Contracting (Jim)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comfort Windows And Doors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novahaus Development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NA Contracting (Nelio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Golden Peak Construction (Edwin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lumber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central Fairbank (Bruno)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KOTT (Jon Stark)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alps Roofing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA Roofing (Jason)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ebi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime Seal Roofing Systems (Ellery)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Honest Roofing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SM Cladding (Milos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roof + Siding + Skylight Combo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety Roofing (Elvis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HVAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ideal Heating (Leena)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MiTech HVAC (Mikel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sentral HVAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMS HVAC</t>
+  </si>
+  <si>
     <t xml:space="preserve">FoamIt (Nadia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bid #13. Milan Insulation $2,372 (#54) also in.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target $3,200.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stephenson's Rentals + United (toilet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scaffold $1,446 + hoist $3,731 + bins $2,800 (Stephenson's #66) + toilet $1,000 (United #64) + boom/deliveries $1,500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Built up from the quoted monthly rates. JobTread shows $2,539 / $2,928, which are not the full rental.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ridge raise + re-shingle (if required)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Framer + Prime Seal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contract: raise front ridge as required. Not priced by any trade yet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allowance. Get it priced as a separate line; drop to $0 if La Vecchia confirms it is not needed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skylight unit + install (flat, den)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RONA unit + framer install</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RONA $289 (#61) + $250 install allowance. Opening framed, curb waterproofed by roofer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm the flat skylight is in the contract price (added May 24).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Winter protection / temporary heat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PalmView</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allowance: tarps, poly, temporary heat while the roof is open in Jan to Feb</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allowance. Remove if demo moves to spring.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">At quoted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">At required (negotiated)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target markup on cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scope check (Oct 25)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aluminum: new roof drainage, coping and existing eavestrough tie-ins carried by the roofer; soffit, fascia and window capping in Baz's siding scope.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Window count: Aryan's scope says 6 window openings; drawings, Baz and the other framers say 4. Confirm before framing award and window order.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrical: HVAC Option 2 needs a 15A double-pole breaker, not the 30A in Fabiano's scope. Update his work order (small credit).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Side-wall cladding: designer to confirm vinyl is allowed at the side wall (limiting distance) before Baz orders.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Building permit fee: confirm whether the client pays the City directly (they paid the zoning fee).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not in base cost: windows (supply + install) and client finish materials (hardwood, interior doors, hardware). Add-ons priced separately.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">439 Manning Ave: Bid Leveling Inputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellow cells are the levers. Change them and every tab updates. Blue = typed-in number, black = formula, green = pulled from another tab.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Input</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source / note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contract sell: 2.0 Rear Addition (pre-HST)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tender Package, Margin Check (from invoice #22288). Excludes design fees and add-ons.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target markup on cost (SOP Step 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tendering SOP: cost target = contract sell / 1.35.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabiano General Works price (negotiated target)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raff's negotiation target, Oct 22. Fabiano quoted $30,500 for General Works (JobTread bid #15). Change to the agreed number.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Does Fabiano's price include demolition? (Yes/No)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabiano priced demo as a separate line ($7,400), per the work order.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demolition cost if separate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabiano demo line, JobTread bid #15 (Oct 22). Doctor Demo still pending.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roof + siding option (Split / Safety)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Split</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Split = lowest flat roof bid + lowest siding bid (now Prime Seal $5,900 + Baz $7,900). Safety = Safety Roofing combo $20,580 (siding, flat roof and skylight).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Construction contingency (% of cost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tender Package: 10% budget reserve.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tender Package P2 provisional / change order risk.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All Manning Bid Requests (from JobTread, Oct 25, 2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amounts are the cost entered on each JobTread bid request. HST treatment not confirmed. To add a bid, insert a row above the last one and copy column E down.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vendor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amount ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lookup key (formula)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JobTread #</t>
-  </si>
-  <si>
-    <t xml:space="preserve">General Works + Demo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renomar Inc (Olimpiu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approved</t>
-  </si>
-  <si>
-    <t xml:space="preserve">General Works (excl. demo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demolition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doctor Demo (Roman)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bradley Demolition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Declined</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Universal Impact Services</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Framing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Age Construction (Mario)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bogdan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JB Contracting (Jim)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comfort Windows And Doors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Novahaus Development</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NA Contracting (Nelio)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Golden Peak Construction (Edwin)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lumber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Central Fairbank (Bruno)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KOTT (Jon Stark)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alps Roofing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CA Roofing (Jason)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ebi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prime Seal Roofing Systems (Ellery)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Honest Roofing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Siding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SM Cladding (Milos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roof + Siding + Skylight Combo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Safety Roofing (Elvis)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HVAC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ideal Heating (Leena)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MiTech HVAC (Mikel)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sentral HVAC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MMS HVAC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Milan Insulation (Andy Cruz)</t>
   </si>
   <si>
     <t xml:space="preserve">Site Services</t>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">'Leveling 2.0'!$F$22</f>
-        <v>86516</v>
+        <v>85687.8</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">'Leveling 2.0'!$E$22</f>
-        <v>95012.69</v>
+        <v>94023.99</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B28" s="9" t="n">
         <f aca="false">'Leveling 2.0'!$F$25</f>
-        <v>0.241553432103095</v>
+        <v>0.248813886210222</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">'Leveling 2.0'!$E$25</f>
-        <v>0.167066801087052</v>
+        <v>0.175734285964758</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">'Leveling 2.0'!$F$34</f>
-        <v>0.121876041027439</v>
+        <v>0.129862540545279</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -4920,7 +4920,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="42" t="s">
         <v>167</v>
       </c>
@@ -4934,19 +4934,20 @@
         <v>3430</v>
       </c>
       <c r="E11" s="8" t="n">
-        <f aca="false">'All Bids'!$D$34</f>
-        <v>3360.5</v>
-      </c>
-      <c r="F11" s="43" t="n">
-        <v>3200</v>
+        <f aca="false">'All Bids'!$D$35</f>
+        <v>2371.8</v>
+      </c>
+      <c r="F11" s="36" t="n">
+        <f aca="false">E11</f>
+        <v>2371.8</v>
       </c>
       <c r="G11" s="26" t="n">
         <f aca="false">E11-F11</f>
-        <v>160.5</v>
+        <v>0</v>
       </c>
       <c r="H11" s="26" t="n">
         <f aca="false">F11-D11</f>
-        <v>-230</v>
+        <v>-1058.2</v>
       </c>
       <c r="I11" s="42" t="s">
         <v>235</v>
@@ -5093,19 +5094,19 @@
       </c>
       <c r="E16" s="31" t="n">
         <f aca="false">SUM(E5:E15)</f>
-        <v>95012.69</v>
+        <v>94023.99</v>
       </c>
       <c r="F16" s="31" t="n">
         <f aca="false">SUM(F5:F15)</f>
-        <v>86516</v>
+        <v>85687.8</v>
       </c>
       <c r="G16" s="31" t="n">
         <f aca="false">SUM(G5:G15)</f>
-        <v>8496.69</v>
+        <v>8336.19</v>
       </c>
       <c r="H16" s="31" t="n">
         <f aca="false">SUM(H5:H15)</f>
-        <v>-28883</v>
+        <v>-29711.2</v>
       </c>
       <c r="I16" s="29"/>
     </row>
@@ -5203,11 +5204,11 @@
       <c r="D22" s="2"/>
       <c r="E22" s="36" t="n">
         <f aca="false">E16</f>
-        <v>95012.69</v>
+        <v>94023.99</v>
       </c>
       <c r="F22" s="36" t="n">
         <f aca="false">F16</f>
-        <v>86516</v>
+        <v>85687.8</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -5222,11 +5223,11 @@
       <c r="D23" s="2"/>
       <c r="E23" s="37" t="n">
         <f aca="false">E22-E21</f>
-        <v>10516.3937037037</v>
+        <v>9527.69370370371</v>
       </c>
       <c r="F23" s="37" t="n">
         <f aca="false">F22-F21</f>
-        <v>2019.70370370371</v>
+        <v>1191.50370370371</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
@@ -5241,11 +5242,11 @@
       <c r="D24" s="2"/>
       <c r="E24" s="37" t="n">
         <f aca="false">E19-E22</f>
-        <v>19057.31</v>
+        <v>20046.01</v>
       </c>
       <c r="F24" s="37" t="n">
         <f aca="false">F19-F22</f>
-        <v>27554</v>
+        <v>28382.2</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -5260,11 +5261,11 @@
       <c r="D25" s="2"/>
       <c r="E25" s="38" t="n">
         <f aca="false">IF(E19=0,0,E24/E19)</f>
-        <v>0.167066801087052</v>
+        <v>0.175734285964758</v>
       </c>
       <c r="F25" s="38" t="n">
         <f aca="false">IF(F19=0,0,F24/F19)</f>
-        <v>0.241553432103095</v>
+        <v>0.248813886210222</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -5279,11 +5280,11 @@
       <c r="D26" s="2"/>
       <c r="E26" s="38" t="n">
         <f aca="false">IF(E22=0,0,E24/E22)</f>
-        <v>0.200576470364117</v>
+        <v>0.21320101391145</v>
       </c>
       <c r="F26" s="38" t="n">
         <f aca="false">IF(F22=0,0,F24/F22)</f>
-        <v>0.318484442184105</v>
+        <v>0.331228016123649</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -5341,11 +5342,11 @@
       <c r="D30" s="2"/>
       <c r="E30" s="36" t="n">
         <f aca="false">E22*Inputs!$B$11</f>
-        <v>9501.269</v>
+        <v>9402.399</v>
       </c>
       <c r="F30" s="36" t="n">
         <f aca="false">F22*Inputs!$B$11</f>
-        <v>8651.6</v>
+        <v>8568.78</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -5379,11 +5380,11 @@
       <c r="D32" s="2"/>
       <c r="E32" s="37" t="n">
         <f aca="false">E22+E30+E31</f>
-        <v>109513.959</v>
+        <v>108426.389</v>
       </c>
       <c r="F32" s="37" t="n">
         <f aca="false">F22+F30+F31</f>
-        <v>100167.6</v>
+        <v>99256.58</v>
       </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
@@ -5398,11 +5399,11 @@
       <c r="D33" s="2"/>
       <c r="E33" s="36" t="n">
         <f aca="false">E19-E32</f>
-        <v>4556.041</v>
+        <v>5643.61099999999</v>
       </c>
       <c r="F33" s="36" t="n">
         <f aca="false">F19-F32</f>
-        <v>13902.4</v>
+        <v>14813.42</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -5417,11 +5418,11 @@
       <c r="D34" s="2"/>
       <c r="E34" s="38" t="n">
         <f aca="false">IF(E19=0,0,E33/E19)</f>
-        <v>0.0399407469097922</v>
+        <v>0.0494749802752695</v>
       </c>
       <c r="F34" s="38" t="n">
         <f aca="false">IF(F19=0,0,F33/F19)</f>
-        <v>0.121876041027439</v>
+        <v>0.129862540545279</v>
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
@@ -6391,7 +6392,7 @@
         <v>167</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>233</v>
+        <v>324</v>
       </c>
       <c r="C34" s="21" t="s">
         <v>291</v>
@@ -6412,7 +6413,7 @@
         <v>167</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>324</v>
+        <v>233</v>
       </c>
       <c r="C35" s="21" t="s">
         <v>291</v>

</xml_diff>